<commit_message>
Theme and society topic pages: 23 new pages, pilot refreshed, 102 pages in pages.xlsx
- content/pages-drafts/: Theme pages batch A and B (18 themes), Society topic pages (Equality, Tolerance, Work and wealth, War and peace, Law and rights); pilot re-exported (Friendship and kindness, path-name labels)
- content/pages.xlsx: 102 pages (59 thinkers, 4 texts, 12 paths, 27 topics); each of the 21 themes has exactly one page
- tools/import_pages.py: a re-imported doc drops pages it no longer contains
- exports/handover-thinker-pages-2026-10-29.md: theme and society pages, theme-to-page check

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XtUBtsHEVvdoDDiuP88LhW
</commit_message>
<xml_diff>
--- a/content/pages.xlsx
+++ b/content/pages.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD80"/>
+  <dimension ref="A1:AD103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7362,7 +7362,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>topic-democracy</t>
+          <t>topic-beauty-and-art</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -7372,30 +7372,26 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Democracy</t>
+          <t>Beauty and art</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>**Democracy** · hand-picked thoughts · [n] thoughts so far</t>
+          <t>**Beauty and art** · theme: Beauty and art · [n] thoughts so far</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr"/>
-      <c r="F77" s="2" t="inlineStr"/>
-      <c r="G77" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H77" s="2" t="inlineStr">
-        <is>
-          <t>128,130,131,160,201,442,617,621</t>
-        </is>
-      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Beauty and art</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr"/>
+      <c r="H77" s="2" t="inlineStr"/>
       <c r="I77" s="2" t="inlineStr"/>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>Should the people rule, and what keeps the many from going wrong?</t>
+          <t>Is beauty out there, or in the eye of the beholder?</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7410,11 +7406,10 @@
       <c r="T77" s="2" t="inlineStr"/>
       <c r="U77" s="2" t="inlineStr">
         <is>
-          <t>**Athens and Plato (Ancient Greece).** Democracy began in Athens around 508 BCE. Citizens voted directly in an assembly, and many officials and jurors were chosen by lot. But only adult male citizens took part, perhaps one person in five or fewer: women, slaves, and foreigners were left out.
-Plato did not trust it. In his parable of the ship, the sailors fight over the helm, while the true pilot, who knows the winds and the stars, is mocked as a stargazer. He had seen a democratic jury sentence his teacher Socrates to death in 399 BCE.
-**Aristotle (Ancient Greece).** Aristotle was more open. A citizen, for him, is someone who takes turns governing and being governed, and a crowd can judge many things better than one person. Still, he feared rule by the many could turn into mob rule. He preferred a mixed government, held steady by a strong middle class.
-**Laozi (Taoists).** The *Tao Te Ching* looks at power from below. The best rulers are those the people hardly notice; worse ones are loved, then feared, then despised. Good government works quietly and lets people feel they did things themselves.
-**Rousseau and Mill (the Enlightenment and after).** Rousseau put the people at the heart of the state: when citizens stop caring about public affairs, the state is lost. Mill, a century later, saw a new danger. A majority can be a tyrant too, and silencing even one person who disagrees harms everyone. The phrase "tyranny of the majority" comes from Alexis de Tocqueville; Mill made it famous.</t>
+          <t>**Kenkō and Okakura (Japanese Aesthetics).** The Japanese writers love what is unfinished. Kenkō thought it better to leave a little imperfection, since perfect uniformity is dull. In *The Book of Tea*, Okakura says true beauty is found by the one who completes the incomplete in their own mind: what is left unsaid gives the viewer a part to play.
+**Hume (Enlightenment Ethics).** Hume started from the view that beauty is no quality in things, but exists in the mind that looks at them. Yet he did not leave it there. Some judgements are better than others, he argued, and the standard of taste is the shared verdict of rare, experienced, unprejudiced critics. Studying beauty, he added, softens the temper.
+**Laozi (Taoism).** The *Tao Te Ching* sees a hidden cost in naming beauty: as soon as everyone knows what is beautiful, they also know what is ugly. Each idea brings its opposite with it.
+**Nietzsche and Emerson (Existential Thought, Humanists and Essayists).** For Nietzsche, the greatest art is to "give style" to your own character, shaping strengths and weaknesses into one whole. Emerson saw in every work of genius our own rejected thoughts, coming back to us with a kind of borrowed majesty.</t>
         </is>
       </c>
       <c r="V77" s="2" t="inlineStr"/>
@@ -7422,16 +7417,14 @@
       <c r="X77" s="2" t="inlineStr"/>
       <c r="Y77" s="2" t="inlineStr">
         <is>
-          <t>None of them trusts power without limits, whoever holds it. They split on whether ordinary people can be trusted to judge. Plato said no, Aristotle said often, and Mill said yes, but only with free speech protecting the few who disagree.</t>
+          <t>All of them link beauty to the person who sees it, not only to the object. They differ on how far. Hume searches for a standard that lets us say some tastes are better; the Japanese writers make the viewer a partner in the work; Nietzsche turns the art inward, onto how we shape our lives.</t>
         </is>
       </c>
       <c r="Z77" s="2" t="inlineStr"/>
       <c r="AA77" s="2" t="inlineStr">
         <is>
-          <t>- Wikipedia, "Athenian democracy": https://en.wikipedia.org/wiki/Athenian_democracy
-- Stanford Encyclopedia of Philosophy, "Aristotle's Political Theory": https://plato.stanford.edu/entries/aristotle-politics/ · "Plato's Ethics and Politics in The Republic": https://plato.stanford.edu/entries/plato-ethics-politics/ · Plato, Republic, Book VI (Jowett translation, Project Gutenberg): https://www.gutenberg.org/ebooks/1497
-- Wikipedia, "Tyranny of the majority": https://en.wikipedia.org/wiki/Tyranny_of_the_majority
-- The app's thoughts listed above, with their sources</t>
+          <t>- Stanford Encyclopedia of Philosophy, "Hume's Aesthetics": https://plato.stanford.edu/entries/hume-aesthetics/
+- The app's thoughts #177, #188, #259, #264, #421, #525, #533, and #534, with their sources</t>
         </is>
       </c>
       <c r="AB77" s="2" t="inlineStr">
@@ -7441,7 +7434,7 @@
       </c>
       <c r="AC77" s="2" t="inlineStr">
         <is>
-          <t>Thinker and topic pages pilot</t>
+          <t>Theme pages, batch B</t>
         </is>
       </c>
       <c r="AD77" s="2" t="inlineStr"/>
@@ -7449,7 +7442,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>topic-freedom</t>
+          <t>topic-change-and-impermanence</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -7459,34 +7452,26 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Freedom</t>
+          <t>Change and impermanence</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>**Freedom** · theme: Freedom, choice, and intention, plus hand-picked thoughts · [n] thoughts so far</t>
+          <t>**Change and impermanence** · theme: Change and impermanence · [n] thoughts so far</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr"/>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Freedom, choice, and intention</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>179,193,294,485,621,625</t>
-        </is>
-      </c>
+          <t>Change and impermanence</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr"/>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>Are you free when nobody stops you, or when you master yourself?</t>
+          <t>Everything changes, so how should we live with it?</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr"/>
@@ -7501,10 +7486,10 @@
       <c r="T78" s="2" t="inlineStr"/>
       <c r="U78" s="2" t="inlineStr">
         <is>
-          <t>**The Stoics and the East: freedom inside.** Epictetus taught that some things are in our power and others are not; freedom starts with knowing the difference. Spinoza called being ruled by your emotions a kind of bondage. Confucius said an army can lose its general, but nobody can take away the will of an ordinary person. Here, freedom is something no prison can remove.
-**Mill: freedom from others.** For Mill, the only freedom worth the name is to pursue your own good in your own way, as long as you do not stop others from doing the same. Over your own body and mind, you rule. Society may step in only to prevent harm to others. Yet Mill limited this to people "in the maturity of their faculties", and in the same chapter he called despotism legitimate over people he called "barbarians", if it improved them.
-**Rousseau and Locke: freedom with others.** Rousseau opens *The Social Contract* by saying people are born free and everywhere in chains. His answer is not fewer laws, but laws the people make together. Locke agrees that law, done well, does not restrain freedom but protects and enlarges it.
-**Wollstonecraft and Fuller: freedom for whom?** Both asked why freedom stopped at men. Wollstonecraft argued that blind obedience is what power wants, and education is the way out. Fuller wanted every path open to women as freely as to men.</t>
+          <t>**Heraclitus and Lucretius (Classical Greek Philosophy, Epicureanism).** Heraclitus said you cannot step into the same river twice, because new water is always flowing. Lucretius saw the same motion in matter itself: nothing comes from nothing, and nothing returns to nothing; things only break apart and form again.
+**The Dhammapada (Buddhist Philosophy).** For the *Dhammapada*, seeing clearly that all created things pass away is itself a path out of suffering. We suffer when we cling to what cannot last.
+**Epictetus and Marcus Aurelius (Stoicism).** Epictetus advised never saying "I have lost it", only "I have given it back": a child, a wife, an estate were only lent to us. Marcus Aurelius put it in five words: the universe is transformation.
+**Kenkō and Okakura (Japanese Aesthetics).** The Japanese writers find beauty in passing things. Kenkō asks whether we should look at the moon only when it is full, or at flowers only in full bloom. Okakura invites us to "dream of evanescence".</t>
         </is>
       </c>
       <c r="V78" s="2" t="inlineStr"/>
@@ -7512,15 +7497,13 @@
       <c r="X78" s="2" t="inlineStr"/>
       <c r="Y78" s="2" t="inlineStr">
         <is>
-          <t>In 1958 the philosopher Isaiah Berlin named the split: "negative" freedom, being left alone, and "positive" freedom, being in control of your own life. Mill stands for the first, Rousseau for the second. Berlin warned that the second can be abused, when rulers claim to force people towards their "real" good. Liberals, in turn, would not call the Stoics' inner freedom real freedom at all.</t>
+          <t>All of them start from the same fact: nothing stays as it is. They differ on what to do with it. The Stoics accept it calmly; the Buddhist texts let go; the Japanese writers find beauty in it; Nietzsche goes further and welcomes change as the way we become new.</t>
         </is>
       </c>
       <c r="Z78" s="2" t="inlineStr"/>
       <c r="AA78" s="2" t="inlineStr">
         <is>
-          <t>- Stanford Encyclopedia of Philosophy, "Positive and Negative Liberty": https://plato.stanford.edu/entries/liberty-positive-negative/
-- John Stuart Mill, *On Liberty* (1859), chapter I (Project Gutenberg): https://www.gutenberg.org/ebooks/34901 · Wikipedia, "Negative liberty": https://en.wikipedia.org/wiki/Negative_liberty · Stanford Encyclopedia of Philosophy, 2014 version of the same entry (on the Stoics): https://plato.stanford.edu/archives/sum2014/entries/liberty-positive-negative/
-- The app's thoughts #15, #42, #168, #197, #198, and the others listed above, with their sources</t>
+          <t>- The app's thoughts #18, #33, #88, #121, #209, #345, #515, #517, and #529, with their sources</t>
         </is>
       </c>
       <c r="AB78" s="2" t="inlineStr">
@@ -7530,7 +7513,7 @@
       </c>
       <c r="AC78" s="2" t="inlineStr">
         <is>
-          <t>Thinker and topic pages pilot</t>
+          <t>Theme pages, batch A</t>
         </is>
       </c>
       <c r="AD78" s="2" t="inlineStr"/>
@@ -7538,7 +7521,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>topic-friendship</t>
+          <t>topic-character-and-virtue</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -7548,18 +7531,18 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Friendship</t>
+          <t>Character and virtue</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>**Friendship** · theme: Friendship and kindness · [n] thoughts so far</t>
+          <t>**Character and virtue** · theme: Character and virtue · [n] thoughts so far</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr"/>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Friendship and kindness</t>
+          <t>Character and virtue</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr"/>
@@ -7567,7 +7550,7 @@
       <c r="I79" s="2" t="inlineStr"/>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>What makes someone a real friend, and why do we need them?</t>
+          <t>What makes a person good, and can you become one?</t>
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr"/>
@@ -7582,10 +7565,10 @@
       <c r="T79" s="2" t="inlineStr"/>
       <c r="U79" s="2" t="inlineStr">
         <is>
-          <t>**Aristotle (Ancient Greece).** He saw three kinds of friendship: for usefulness, for pleasure, and for character. The first two fade when the use or the fun ends. Only the third lasts, because each friend loves who the other is. Such a friend, he says, is "another self", and good friends make each other better. He thought nobody would choose a life without friends, even with everything else.
-**Epicurus (Ancient Greece).** For Epicurus, friendship was the greatest help to a happy life, worth more than wealth or power. He lived it: his school, the Garden, was a community of friends outside politics, who shared meals and celebrations, and it welcomed women as students.
-**Confucius (Ancient China).** Friends help each other grow in virtue. A good friend tells you honestly when you are wrong, and does it with tact. But if the friend will not listen, you stop, rather than lose the friendship.
-**Montaigne (the Humanists).** After his friend Étienne de La Boétie died young, Montaigne wrote that true friendship cannot be explained: it happens between these two people, and no others. He believed such a friendship is so complete that a person can have only one, and that it is very rare. In the same essay he says women had never reached this kind of friendship, a view common among writers of his time.</t>
+          <t>**Aristotle (Classical Greek Philosophy).** Virtue, for Aristotle, is a settled trait of character, and you build it the way you learn a craft: by doing. We become just by doing just acts and brave by doing brave ones. Each virtue sits between two extremes, like courage between cowardice and recklessness. Hitting that middle point is hard, and it takes practical wisdom.
+**Confucius (Confucianism).** People start out much alike, Confucius said, and practice makes them grow far apart. The ideal is the "superior man", who asks a lot of himself and little of others, and who leads by example rather than by orders. Virtue is never lonely: whoever practises it will find neighbours.
+**The Dhammapada (Buddhist Philosophy).** The *Dhammapada* puts the work in each person's hands: by oneself evil is done, and by oneself it is left undone. Small good acts add up, like a water jar filling drop by drop. Anger is overcome by love, and evil by good.
+**Kant (Enlightenment Ethics).** Kant moved the focus from character to the will. Talents, courage, and even happiness can be used for bad ends; only a good will is good without qualification. Morality, he said, is not about how to be happy, but how to become worthy of happiness.</t>
         </is>
       </c>
       <c r="V79" s="2" t="inlineStr"/>
@@ -7593,17 +7576,15 @@
       <c r="X79" s="2" t="inlineStr"/>
       <c r="Y79" s="2" t="inlineStr">
         <is>
-          <t>All four see friendship as one of the best things in life, and all link it to becoming a better person. They differ on numbers and reasons. Epicurus spoke openly of the safety and pleasure friends give; Aristotle cared most about friends valued for themselves; Montaigne thought the deepest kind happens only once. Nietzsche adds a sharper voice: a true friend should also challenge you.</t>
+          <t>All four say goodness takes effort and is not simply given at birth. They split on where it lives. For Aristotle and Confucius, it is a character shaped by long practice and good company; for Kant, it is the intention behind each act, done out of duty. Virtue ethics, the tradition of Aristotle and Confucius, faded in the West after the Enlightenment and returned in the late 1950s.</t>
         </is>
       </c>
       <c r="Z79" s="2" t="inlineStr"/>
       <c r="AA79" s="2" t="inlineStr">
         <is>
-          <t>- Stanford Encyclopedia of Philosophy, "Friendship": https://plato.stanford.edu/entries/friendship/
-- Wikipedia, "Epicurus": https://en.wikipedia.org/wiki/Epicurus
-- Cambridge University Library, "Of friendship" (Montaigne exhibition): https://wwwe.lib.cam.ac.uk/CUL/exhibitions/Montaigne/c3.html
-- Montaigne, "Of Friendship", Cotton translation (HyperEssays): https://hyperessays.net/essays/on-friendship/ · Wikipedia, "Michel de Montaigne": https://en.wikipedia.org/wiki/Michel_de_Montaigne
-- The app's thoughts #58, #112, #115, #117, #211, #280, #502, and #503, with their sources</t>
+          <t>- Stanford Encyclopedia of Philosophy, "Virtue Ethics": https://plato.stanford.edu/entries/ethics-virtue/
+- Stanford Encyclopedia of Philosophy, "Kant's Moral Philosophy": https://plato.stanford.edu/entries/kant-moral/ · "Confucius": https://plato.stanford.edu/entries/confucius/
+- The app's thoughts #109, #113, #119, #154, #155, #208, #328, #333, #339, #357, #475, #487, #492, #495, and #504, with their sources</t>
         </is>
       </c>
       <c r="AB79" s="2" t="inlineStr">
@@ -7613,7 +7594,7 @@
       </c>
       <c r="AC79" s="2" t="inlineStr">
         <is>
-          <t>Thinker and topic pages pilot</t>
+          <t>Theme pages, batch A</t>
         </is>
       </c>
       <c r="AD79" s="2" t="inlineStr"/>
@@ -7621,7 +7602,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>topic-justice</t>
+          <t>topic-death-and-mortality</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -7631,30 +7612,26 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Justice</t>
+          <t>Death and mortality</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>**Justice** · theme: Justice, power, and leadership · [n] thoughts so far</t>
+          <t>**Death and mortality** · theme: Death and mortality · [n] thoughts so far</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Justice, power, and leadership</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>Death and mortality</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr"/>
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr"/>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>What do we owe each other, and who decides?</t>
+          <t>Should we think about death, and can we stop fearing it?</t>
         </is>
       </c>
       <c r="K80" s="2" t="inlineStr"/>
@@ -7669,10 +7646,10 @@
       <c r="T80" s="2" t="inlineStr"/>
       <c r="U80" s="2" t="inlineStr">
         <is>
-          <t>**Plato and Socrates (Ancient Greece).** In Plato's *Republic*, a character called Thrasymachus says justice is simply what serves the strong. Plato's answer is that justice is a kind of harmony: each part of a person, or of a city, doing its proper job. His teacher Socrates went further. He said it is better to suffer an injustice than to do one, and that we should never return harm for harm.
-**Aristotle (Ancient Greece).** For Aristotle, justice means giving people what they deserve, and good laws are reason without passion. A citizen is someone who takes turns ruling and being ruled. Yet the same book, the *Politics*, argues that some people are slaves by nature. Centuries later, this idea was used to defend the enslavement of Native Americans.
-**Epicurus (Ancient Greece).** Epicurus saw no justice written into nature. For him, justice is an agreement between people not to harm each other, and it can change from place to place. It still matters to the individual: the just person lives with the most peace of mind.
-**Confucius (Ancient China).** Justice begins with the people who lead. A ruler who acts rightly will be followed without needing many orders. When someone wrongs you, answer with justice, not with kindness or revenge. In classical Confucian thought, justice was a personal and public virtue, not a matter of law or equal rights.</t>
+          <t>**Epicurus and Lucretius (Epicureanism).** Epicurus argued that death is nothing to us: where death is, we are not, and where we are, death is not. Lucretius asked why we should not leave life like a guest leaving a banquet, full and content. On the day he died, in great pain, Epicurus wrote to a friend that the memory of their conversations outweighed it all.
+**Marcus Aurelius and Montaigne (Stoicism, Humanists and Essayists).** Marcus Aurelius reminded himself not to act as if he had ten thousand years. Montaigne took an old saying for an essay title: to study philosophy is to learn to die. Whoever has learned to die, he said, has unlearned how to be a slave.
+**Zhuangzi (Taoism).** When Zhuangzi's wife died, a friend found him beating on a bowl and singing. He had grieved like anyone, he explained, then saw her death as one more change, like spring turning to summer, autumn, and winter. Tagore says something close: death belongs to life as birth does.
+**Omar Khayyam and Kenkō (Persian and Sufi Poetry, Japanese Aesthetics).** For Khayyam, death is a door with no key and a veil no one sees past, so we should make the most of the days we have. Kenkō notes that death does not wait its turn like the seasons; it presses on us from behind.</t>
         </is>
       </c>
       <c r="V80" s="2" t="inlineStr"/>
@@ -7680,28 +7657,1906 @@
       <c r="X80" s="2" t="inlineStr"/>
       <c r="Y80" s="2" t="inlineStr">
         <is>
-          <t>Most agree that justice is about more than rules: it shapes the kind of person you become. They split on where it comes from. For Plato it is part of how things should be; for Epicurus, and later for social contract thinkers like Rousseau, it is something people agree on. Modern debates add new questions the ancients rarely asked, such as how fair inequality can be, as in John Rawls's "veil of ignorance", or whether punishment should aim to repair harm.</t>
+          <t>Most of them say that facing death honestly makes life clearer and fear smaller. They split on how much to think about it. Montaigne and the Stoics advise keeping it in mind; Spinoza answered that a free person thinks of death least of all, and that wisdom is a meditation on life.</t>
         </is>
       </c>
       <c r="Z80" s="2" t="inlineStr"/>
       <c r="AA80" s="2" t="inlineStr">
+        <is>
+          <t>- The app's thoughts #4, #59, #73, #75, #170, #277, #387, #437, #520, #582, and #583, with their sources</t>
+        </is>
+      </c>
+      <c r="AB80" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC80" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch B</t>
+        </is>
+      </c>
+      <c r="AD80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>topic-democracy</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Democracy</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>**Democracy** · hand-picked thoughts · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>128,130,131,160,201,442,617,621</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>Should the people rule, and what keeps the many from going wrong?</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr"/>
+      <c r="L81" s="2" t="inlineStr"/>
+      <c r="M81" s="2" t="inlineStr"/>
+      <c r="N81" s="2" t="inlineStr"/>
+      <c r="O81" s="2" t="inlineStr"/>
+      <c r="P81" s="2" t="inlineStr"/>
+      <c r="Q81" s="2" t="inlineStr"/>
+      <c r="R81" s="2" t="inlineStr"/>
+      <c r="S81" s="2" t="inlineStr"/>
+      <c r="T81" s="2" t="inlineStr"/>
+      <c r="U81" s="2" t="inlineStr">
+        <is>
+          <t>**Athens and Plato (Classical Greek Philosophy).** Democracy began in Athens around 508 BCE. Citizens voted directly in an assembly, and many officials and jurors were chosen by lot. But only adult male citizens took part, perhaps one person in five or fewer: women, slaves, and foreigners were left out.
+Plato did not trust it. In his parable of the ship, the sailors fight over the helm, while the true pilot, who knows the winds and the stars, is mocked as a stargazer. He had seen a democratic jury sentence his teacher Socrates to death in 399 BCE.
+**Aristotle (Classical Greek Philosophy).** Aristotle was more open. A citizen, for him, is someone who takes turns governing and being governed, and a crowd can judge many things better than one person. Still, he feared rule by the many could turn into mob rule. He preferred a mixed government, held steady by a strong middle class.
+**Laozi (Taoism).** The *Tao Te Ching* looks at power from below. The best rulers are those the people hardly notice; worse ones are loved, then feared, then despised. Good government works quietly and lets people feel they did things themselves.
+**Rousseau and Mill (Enlightenment Ethics).** Rousseau put the people at the heart of the state: when citizens stop caring about public affairs, the state is lost. Mill, a century later, saw a new danger. A majority can be a tyrant too, and silencing even one person who disagrees harms everyone. The phrase "tyranny of the majority" comes from Alexis de Tocqueville; Mill made it famous.</t>
+        </is>
+      </c>
+      <c r="V81" s="2" t="inlineStr"/>
+      <c r="W81" s="2" t="inlineStr"/>
+      <c r="X81" s="2" t="inlineStr"/>
+      <c r="Y81" s="2" t="inlineStr">
+        <is>
+          <t>None of them trusts power without limits, whoever holds it. They split on whether ordinary people can be trusted to judge. Plato said no, Aristotle said often, and Mill said yes, but only with free speech protecting the few who disagree.</t>
+        </is>
+      </c>
+      <c r="Z81" s="2" t="inlineStr"/>
+      <c r="AA81" s="2" t="inlineStr">
+        <is>
+          <t>- Wikipedia, "Athenian democracy": https://en.wikipedia.org/wiki/Athenian_democracy
+- Stanford Encyclopedia of Philosophy, "Aristotle's Political Theory": https://plato.stanford.edu/entries/aristotle-politics/ · "Plato's Ethics and Politics in The Republic": https://plato.stanford.edu/entries/plato-ethics-politics/ · Plato, Republic, Book VI (Jowett translation, Project Gutenberg): https://www.gutenberg.org/ebooks/1497
+- Wikipedia, "Tyranny of the majority": https://en.wikipedia.org/wiki/Tyranny_of_the_majority
+- The app's thoughts listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="AB81" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC81" s="2" t="inlineStr">
+        <is>
+          <t>Thinker and topic pages pilot</t>
+        </is>
+      </c>
+      <c r="AD81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>topic-desire-and-simplicity</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Desire and simplicity</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>**Desire and simplicity** · theme: Desire and simplicity · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Desire and simplicity</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr"/>
+      <c r="H82" s="2" t="inlineStr"/>
+      <c r="I82" s="2" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>Would we be happier wanting less?</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr"/>
+      <c r="M82" s="2" t="inlineStr"/>
+      <c r="N82" s="2" t="inlineStr"/>
+      <c r="O82" s="2" t="inlineStr"/>
+      <c r="P82" s="2" t="inlineStr"/>
+      <c r="Q82" s="2" t="inlineStr"/>
+      <c r="R82" s="2" t="inlineStr"/>
+      <c r="S82" s="2" t="inlineStr"/>
+      <c r="T82" s="2" t="inlineStr"/>
+      <c r="U82" s="2" t="inlineStr">
+        <is>
+          <t>**Epicurus (Epicureanism).** Epicurus sorted desires into three kinds: natural and necessary, like drinking when thirsty; natural but not necessary, like costly food; and neither, like statues in your honour. The first are easy to satisfy; the last have no limit. Nature's wealth, he said, is small and easy to get.
+**Marcus Aurelius, Epictetus, and Seneca (Stoicism).** Marcus Aurelius advised doing few things if you want peace of mind. Epictetus put it more bluntly: don't admire your clothes, and you won't be angry with the thief. Seneca noted that we fear everything as if we were mortal, and want everything as if we would live forever.
+**The Bhagavad Gita and the Dhammapada (Indian Philosophy, Buddhist Philosophy).** The *Gita* traces a chain: dwelling on things breeds attachment, attachment breeds desire, and desire breeds anger. Its answer is to act without clinging to the fruits of action. The *Dhammapada* says there is no fire like passion.
+**Laozi and Thoreau (Taoism, Humanists and Essayists).** For Laozi, there is no greater calamity than never being content. Many centuries later, Thoreau went to live by Walden Pond to keep only the essentials of life. His advice: "Simplify, simplify."</t>
+        </is>
+      </c>
+      <c r="V82" s="2" t="inlineStr"/>
+      <c r="W82" s="2" t="inlineStr"/>
+      <c r="X82" s="2" t="inlineStr"/>
+      <c r="Y82" s="2" t="inlineStr">
+        <is>
+          <t>Most agree that endless wanting makes us unhappy, and that it is better to change our desires than the world. Not everyone wants to drop desire, though. Émilie du Châtelet wrote that we are happy only through tastes and passions that are satisfied, and Simone Weil saw desire as what leads the mind.</t>
+        </is>
+      </c>
+      <c r="Z82" s="2" t="inlineStr"/>
+      <c r="AA82" s="2" t="inlineStr">
+        <is>
+          <t>- The app's thoughts #5, #25, #41, #61, #72, #182, #194, #254, #267, #268, #353, #368, #370, and #419, with their sources</t>
+        </is>
+      </c>
+      <c r="AB82" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC82" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch A</t>
+        </is>
+      </c>
+      <c r="AD82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>topic-ego-pride-and-humility</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Ego, pride, and humility</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>**Ego, pride, and humility** · theme: Ego, pride, and humility · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr"/>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Ego, pride, and humility</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr"/>
+      <c r="H83" s="2" t="inlineStr"/>
+      <c r="I83" s="2" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>How much should we think of ourselves?</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr"/>
+      <c r="L83" s="2" t="inlineStr"/>
+      <c r="M83" s="2" t="inlineStr"/>
+      <c r="N83" s="2" t="inlineStr"/>
+      <c r="O83" s="2" t="inlineStr"/>
+      <c r="P83" s="2" t="inlineStr"/>
+      <c r="Q83" s="2" t="inlineStr"/>
+      <c r="R83" s="2" t="inlineStr"/>
+      <c r="S83" s="2" t="inlineStr"/>
+      <c r="T83" s="2" t="inlineStr"/>
+      <c r="U83" s="2" t="inlineStr">
+        <is>
+          <t>**Laozi (Taoism).** The *Tao Te Ching* praises water: it helps everything and settles in the low places others avoid. A cup filled to the brim is hard to carry. Knowing others is clever, it says, but knowing yourself is wisdom.
+**Confucius (Confucianism).** Confucius did not worry about being unknown, only about not knowing others. He noted that people of old studied to improve themselves, while people of his day studied to be seen. His students said he was free of four things, among them stubbornness and egoism.
+**Epictetus (Stoicism).** The first task of anyone who studies philosophy, said Epictetus, is to drop self-conceit, because nobody can learn what they think they already know. He also asked his students to remember how small a part of the whole they are.
+**La Rochefoucauld and Erasmus (Humanists and Essayists).** La Rochefoucauld called self-love the greatest of flatterers, and saw it behind even our virtues. In Erasmus's *Praise of Folly*, Folly herself admits that nothing is sillier than admiring yourself.</t>
+        </is>
+      </c>
+      <c r="V83" s="2" t="inlineStr"/>
+      <c r="W83" s="2" t="inlineStr"/>
+      <c r="X83" s="2" t="inlineStr"/>
+      <c r="Y83" s="2" t="inlineStr">
+        <is>
+          <t>All of them see pride as a blind spot that keeps us from learning and from seeing others clearly. They differ on the cure. Laozi, Confucius, and Epictetus think practice can make us humbler. La Rochefoucauld doubts we ever fully escape self-love; at best we learn to notice it.</t>
+        </is>
+      </c>
+      <c r="Z83" s="2" t="inlineStr"/>
+      <c r="AA83" s="2" t="inlineStr">
+        <is>
+          <t>- The app's thoughts #23, #44, #290, #301, #410, #411, #415, #468, #483, and #490, with their sources</t>
+        </is>
+      </c>
+      <c r="AB83" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC83" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch A</t>
+        </is>
+      </c>
+      <c r="AD83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>topic-equality</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Equality</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>**Equality** · hand-picked thoughts · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr"/>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>128,179,180,295,324,495,621,622</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr"/>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Are people equal, and equal in what?</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr"/>
+      <c r="L84" s="2" t="inlineStr"/>
+      <c r="M84" s="2" t="inlineStr"/>
+      <c r="N84" s="2" t="inlineStr"/>
+      <c r="O84" s="2" t="inlineStr"/>
+      <c r="P84" s="2" t="inlineStr"/>
+      <c r="Q84" s="2" t="inlineStr"/>
+      <c r="R84" s="2" t="inlineStr"/>
+      <c r="S84" s="2" t="inlineStr"/>
+      <c r="T84" s="2" t="inlineStr"/>
+      <c r="U84" s="2" t="inlineStr">
+        <is>
+          <t>**Aristotle (Classical Greek Philosophy).** Aristotle gave the basic rule of fairness: treat like cases alike. Citizens, for him, took turns ruling and being ruled. But he did not think all people were alike: in the same book he argued that some are slaves by nature, an idea later used to defend slavery.
+**The Stoics and Confucius (Stoicism, Confucianism).** Other traditions stressed what we share. The Stoics taught the natural equality of all beings who have reason. Confucius said people are much alike by nature, and grow apart only by practice.
+**Rousseau (Enlightenment Ethics).** Rousseau opens *The Social Contract* by saying people are born free, yet everywhere they are in chains. In his earlier *Discourse on Inequality*, he traced social inequality to the first fences around land: we are lost, he warned, if we forget that the fruits belong to all and the earth to no one.
+**Wollstonecraft and Fuller (Enlightenment Ethics, Humanists and Essayists).** Both asked why equality stopped at men. Wollstonecraft argued that women seemed weaker only because they were denied education. Fuller noted that the self-reliance praised in her was called a fault in most women.</t>
+        </is>
+      </c>
+      <c r="V84" s="2" t="inlineStr"/>
+      <c r="W84" s="2" t="inlineStr"/>
+      <c r="X84" s="2" t="inlineStr"/>
+      <c r="Y84" s="2" t="inlineStr">
+        <is>
+          <t>Until the 18th century, most thinkers assumed people were unequal by nature; the idea of natural rights changed that. Today most agree people are equal in dignity. The open question is equal in what: rights, chances, or results. Rousseau worried about unequal property; Aristotle, even with his blind spots, about treating like cases alike.</t>
+        </is>
+      </c>
+      <c r="Z84" s="2" t="inlineStr"/>
+      <c r="AA84" s="2" t="inlineStr">
+        <is>
+          <t>- Stanford Encyclopedia of Philosophy, "Equality": https://plato.stanford.edu/entries/equality/
+- Wikipedia, "Natural slavery": https://en.wikipedia.org/wiki/Natural_slavery · Stanford Encyclopedia of Philosophy, "Jean Jacques Rousseau": https://plato.stanford.edu/entries/rousseau/
+- The app's thoughts listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="AB84" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC84" s="2" t="inlineStr">
+        <is>
+          <t>Society topic pages</t>
+        </is>
+      </c>
+      <c r="AD84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>topic-freedom</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Freedom</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>**Freedom** · theme: Freedom, choice, and intention, plus hand-picked thoughts · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Freedom, choice, and intention</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>179,193,294,485,621,625</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr"/>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>Are you free when nobody stops you, or when you master yourself?</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr"/>
+      <c r="L85" s="2" t="inlineStr"/>
+      <c r="M85" s="2" t="inlineStr"/>
+      <c r="N85" s="2" t="inlineStr"/>
+      <c r="O85" s="2" t="inlineStr"/>
+      <c r="P85" s="2" t="inlineStr"/>
+      <c r="Q85" s="2" t="inlineStr"/>
+      <c r="R85" s="2" t="inlineStr"/>
+      <c r="S85" s="2" t="inlineStr"/>
+      <c r="T85" s="2" t="inlineStr"/>
+      <c r="U85" s="2" t="inlineStr">
+        <is>
+          <t>**The Stoics and the East: freedom inside.** Epictetus taught that some things are in our power and others are not; freedom starts with knowing the difference. Spinoza called being ruled by your emotions a kind of bondage. Confucius said an army can lose its general, but nobody can take away the will of an ordinary person. Here, freedom is something no prison can remove.
+**Mill: freedom from others.** For Mill, the only freedom worth the name is to pursue your own good in your own way, as long as you do not stop others from doing the same. Over your own body and mind, you rule. Society may step in only to prevent harm to others. Yet Mill limited this to people "in the maturity of their faculties", and in the same chapter he called despotism legitimate over people he called "barbarians", if it improved them.
+**Rousseau and Locke: freedom with others.** Rousseau opens *The Social Contract* by saying people are born free and everywhere in chains. His answer is not fewer laws, but laws the people make together. Locke agrees that law, done well, does not restrain freedom but protects and enlarges it.
+**Wollstonecraft and Fuller: freedom for whom?** Both asked why freedom stopped at men. Wollstonecraft argued that blind obedience is what power wants, and education is the way out. Fuller wanted every path open to women as freely as to men.</t>
+        </is>
+      </c>
+      <c r="V85" s="2" t="inlineStr"/>
+      <c r="W85" s="2" t="inlineStr"/>
+      <c r="X85" s="2" t="inlineStr"/>
+      <c r="Y85" s="2" t="inlineStr">
+        <is>
+          <t>In 1958 the philosopher Isaiah Berlin named the split: "negative" freedom, being left alone, and "positive" freedom, being in control of your own life. Mill stands for the first, Rousseau for the second. Berlin warned that the second can be abused, when rulers claim to force people towards their "real" good. Liberals, in turn, would not call the Stoics' inner freedom real freedom at all.</t>
+        </is>
+      </c>
+      <c r="Z85" s="2" t="inlineStr"/>
+      <c r="AA85" s="2" t="inlineStr">
+        <is>
+          <t>- Stanford Encyclopedia of Philosophy, "Positive and Negative Liberty": https://plato.stanford.edu/entries/liberty-positive-negative/
+- John Stuart Mill, *On Liberty* (1859), chapter I (Project Gutenberg): https://www.gutenberg.org/ebooks/34901 · Wikipedia, "Negative liberty": https://en.wikipedia.org/wiki/Negative_liberty · Stanford Encyclopedia of Philosophy, 2014 version of the same entry (on the Stoics): https://plato.stanford.edu/archives/sum2014/entries/liberty-positive-negative/
+- The app's thoughts #15, #42, #168, #197, #198, and the others listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="AB85" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC85" s="2" t="inlineStr">
+        <is>
+          <t>Thinker and topic pages pilot</t>
+        </is>
+      </c>
+      <c r="AD85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>topic-friendship-and-kindness</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Friendship and kindness</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>**Friendship and kindness** · theme: Friendship and kindness · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Friendship and kindness</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr"/>
+      <c r="H86" s="2" t="inlineStr"/>
+      <c r="I86" s="2" t="inlineStr"/>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>What makes someone a real friend, and why do we need them?</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr"/>
+      <c r="L86" s="2" t="inlineStr"/>
+      <c r="M86" s="2" t="inlineStr"/>
+      <c r="N86" s="2" t="inlineStr"/>
+      <c r="O86" s="2" t="inlineStr"/>
+      <c r="P86" s="2" t="inlineStr"/>
+      <c r="Q86" s="2" t="inlineStr"/>
+      <c r="R86" s="2" t="inlineStr"/>
+      <c r="S86" s="2" t="inlineStr"/>
+      <c r="T86" s="2" t="inlineStr"/>
+      <c r="U86" s="2" t="inlineStr">
+        <is>
+          <t>**Aristotle (Classical Greek Philosophy).** He saw three kinds of friendship: for usefulness, for pleasure, and for character. The first two fade when the use or the fun ends. Only the third lasts, because each friend loves who the other is. Such a friend, he says, is "another self", and good friends make each other better. He thought nobody would choose a life without friends, even with everything else.
+**Epicurus (Epicureanism).** For Epicurus, friendship was the greatest help to a happy life, worth more than wealth or power. He lived it: his school, the Garden, was a community of friends outside politics, who shared meals and celebrations, and it welcomed women as students.
+**Confucius (Confucianism).** Friends help each other grow in virtue. A good friend tells you honestly when you are wrong, and does it with tact. But if the friend will not listen, you stop, rather than lose the friendship.
+**Montaigne (Humanists and Essayists).** After his friend Étienne de La Boétie died young, Montaigne wrote that true friendship cannot be explained: it happens between these two people, and no others. He believed such a friendship is so complete that a person can have only one, and that it is very rare. In the same essay he says women had never reached this kind of friendship, a view common among writers of his time.
+**Mencius (Confucianism).** Kindness, for Mencius, is in everyone from the start. Anyone who suddenly saw a child about to fall into a well would feel alarm and distress, he said, without thinking of reward. That feeling of compassion is the seed of goodness, and it only needs to grow.</t>
+        </is>
+      </c>
+      <c r="V86" s="2" t="inlineStr"/>
+      <c r="W86" s="2" t="inlineStr"/>
+      <c r="X86" s="2" t="inlineStr"/>
+      <c r="Y86" s="2" t="inlineStr">
+        <is>
+          <t>All of them see friendship and kindness as among the best things in life, and link them to becoming a better person. They differ on numbers and reasons. Epicurus spoke openly of the safety and pleasure friends give; Aristotle cared most about friends valued for themselves; Montaigne thought the deepest kind happens only once. Nietzsche adds a sharper voice: a true friend should also challenge you.</t>
+        </is>
+      </c>
+      <c r="Z86" s="2" t="inlineStr"/>
+      <c r="AA86" s="2" t="inlineStr">
+        <is>
+          <t>- Stanford Encyclopedia of Philosophy, "Friendship": https://plato.stanford.edu/entries/friendship/
+- Wikipedia, "Epicurus": https://en.wikipedia.org/wiki/Epicurus
+- Cambridge University Library, "Of friendship" (Montaigne exhibition): https://wwwe.lib.cam.ac.uk/CUL/exhibitions/Montaigne/c3.html
+- Montaigne, "Of Friendship", Cotton translation (HyperEssays): https://hyperessays.net/essays/on-friendship/ · Wikipedia, "Michel de Montaigne": https://en.wikipedia.org/wiki/Michel_de_Montaigne
+- The app's thoughts #58, #112, #115, #117, #211, #280, #502, #503, #511, and #512, with their sources</t>
+        </is>
+      </c>
+      <c r="AB86" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC86" s="2" t="inlineStr">
+        <is>
+          <t>Thinker and topic pages pilot</t>
+        </is>
+      </c>
+      <c r="AD86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>topic-habit-and-practice</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Habit and practice</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>**Habit and practice** · theme: Habit and practice · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Habit and practice</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr"/>
+      <c r="H87" s="2" t="inlineStr"/>
+      <c r="I87" s="2" t="inlineStr"/>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>Are we what we repeatedly do?</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr"/>
+      <c r="L87" s="2" t="inlineStr"/>
+      <c r="M87" s="2" t="inlineStr"/>
+      <c r="N87" s="2" t="inlineStr"/>
+      <c r="O87" s="2" t="inlineStr"/>
+      <c r="P87" s="2" t="inlineStr"/>
+      <c r="Q87" s="2" t="inlineStr"/>
+      <c r="R87" s="2" t="inlineStr"/>
+      <c r="S87" s="2" t="inlineStr"/>
+      <c r="T87" s="2" t="inlineStr"/>
+      <c r="U87" s="2" t="inlineStr">
+        <is>
+          <t>**Epictetus and Aristotle (Stoicism, Classical Greek Philosophy).** If you want to be a good reader, said Epictetus, read; if a writer, write. Nothing great happens suddenly, not even a grape or a fig. Aristotle said the same of goodness: we become just by doing just acts.
+**Confucius (Confucianism).** Confucius compared learning to building a mound, one basket of earth at a time. If you stop one basket short, the stopping is your own doing; if you add one basket, you have moved forward. People start out much alike; practice sets them apart.
+**The Dhammapada (Buddhist Philosophy).** The *Dhammapada* compares training the mind to a fletcher straightening an arrow. Small acts add up, like a water jar filling drop by drop, both for good and for bad. If you do something good, do it again, and take delight in it.
+**Laozi and Zhuangzi (Taoism).** Every great thing starts small: the journey of a thousand li begins with a single step. Zhuangzi's cook has used the same knife for nineteen years. After long practice he no longer sees the whole ox, and works with his mind, following the natural gaps.</t>
+        </is>
+      </c>
+      <c r="V87" s="2" t="inlineStr"/>
+      <c r="W87" s="2" t="inlineStr"/>
+      <c r="X87" s="2" t="inlineStr"/>
+      <c r="Y87" s="2" t="inlineStr">
+        <is>
+          <t>All of them see small, repeated acts as the way a person changes. They differ on the goal. Confucius and Epictetus speak of steady effort; Zhuangzi's cook shows effort turning into ease. Kenkō and Hume add a warning: habits and customs also hold us, and few things are harder to give up.</t>
+        </is>
+      </c>
+      <c r="Z87" s="2" t="inlineStr"/>
+      <c r="AA87" s="2" t="inlineStr">
+        <is>
+          <t>- The app's thoughts #22, #40, #109, #174, #311, #314, #338, #413, #432, #495, #514, and #527, with their sources</t>
+        </is>
+      </c>
+      <c r="AB87" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC87" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch B</t>
+        </is>
+      </c>
+      <c r="AD87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>topic-happiness-and-the-good-life</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Happiness and the good life</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>**Happiness and the good life** · theme: Happiness and the good life · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Happiness and the good life</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr"/>
+      <c r="I88" s="2" t="inlineStr"/>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>What does a good life need, and is happiness the point?</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr"/>
+      <c r="L88" s="2" t="inlineStr"/>
+      <c r="M88" s="2" t="inlineStr"/>
+      <c r="N88" s="2" t="inlineStr"/>
+      <c r="O88" s="2" t="inlineStr"/>
+      <c r="P88" s="2" t="inlineStr"/>
+      <c r="Q88" s="2" t="inlineStr"/>
+      <c r="R88" s="2" t="inlineStr"/>
+      <c r="S88" s="2" t="inlineStr"/>
+      <c r="T88" s="2" t="inlineStr"/>
+      <c r="U88" s="2" t="inlineStr">
+        <is>
+          <t>**Aristotle (Classical Greek Philosophy).** Happiness, for Aristotle, is the one thing we want for its own sake. His word, *eudaimonia*, means living well, or flourishing, not a passing mood. It is judged over a whole life: one swallow does not make a spring, and one good day does not make a happy life.
+**Epicurus (Epicureanism).** Epicurus made pleasure the goal, but not the pleasure of parties and luxury. He meant freedom from pain in the body and fear in the mind. Plain food, once hunger is gone, gives as much pleasure as a feast, and friends are the greatest help of all.
+**Confucius and the Dhammapada (Confucianism, Buddhist Philosophy).** Both find happiness in contentment. Confucius said he could still find joy with coarse rice, water, and his bent arm for a pillow. For the *Dhammapada*, health is the greatest gift and contentment the best riches.
+**Mill and Kant (Enlightenment Ethics).** Mill believed happiness is the goal, but some pleasures are higher than others: better to be Socrates dissatisfied than a fool satisfied. He also warned that happiness comes best on the side, while aiming at something else. Kant answered that morality is not about how to be happy, but how to become worthy of happiness.</t>
+        </is>
+      </c>
+      <c r="V88" s="2" t="inlineStr"/>
+      <c r="W88" s="2" t="inlineStr"/>
+      <c r="X88" s="2" t="inlineStr"/>
+      <c r="Y88" s="2" t="inlineStr">
+        <is>
+          <t>Most agree that happiness is not pleasure piled up, and that wanting less helps. They disagree on whether happiness is the aim of life. For Aristotle, Epicurus, and Mill it is, in different forms; for Kant, doing right comes first, whatever it costs.</t>
+        </is>
+      </c>
+      <c r="Z88" s="2" t="inlineStr"/>
+      <c r="AA88" s="2" t="inlineStr">
+        <is>
+          <t>- Stanford Encyclopedia of Philosophy, "Aristotle's Ethics": https://plato.stanford.edu/entries/aristotle-ethics/
+- The app's thoughts #58, #64, #66, #67, #110, #116, #155, #158, #159, #331, and #479, with their sources</t>
+        </is>
+      </c>
+      <c r="AB88" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC88" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch A</t>
+        </is>
+      </c>
+      <c r="AD88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>topic-justice</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Justice</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>**Justice** · theme: Justice, power, and leadership · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr"/>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Justice, power, and leadership</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr"/>
+      <c r="I89" s="2" t="inlineStr"/>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>What do we owe each other, and who decides?</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr"/>
+      <c r="L89" s="2" t="inlineStr"/>
+      <c r="M89" s="2" t="inlineStr"/>
+      <c r="N89" s="2" t="inlineStr"/>
+      <c r="O89" s="2" t="inlineStr"/>
+      <c r="P89" s="2" t="inlineStr"/>
+      <c r="Q89" s="2" t="inlineStr"/>
+      <c r="R89" s="2" t="inlineStr"/>
+      <c r="S89" s="2" t="inlineStr"/>
+      <c r="T89" s="2" t="inlineStr"/>
+      <c r="U89" s="2" t="inlineStr">
+        <is>
+          <t>**Plato and Socrates (Classical Greek Philosophy).** In Plato's *Republic*, a character called Thrasymachus says justice is simply what serves the strong. Plato's answer is that justice is a kind of harmony: each part of a person, or of a city, doing its proper job. His teacher Socrates went further. He said it is better to suffer an injustice than to do one, and that we should never return harm for harm.
+**Aristotle (Classical Greek Philosophy).** For Aristotle, justice means giving people what they deserve, and good laws are reason without passion. A citizen is someone who takes turns ruling and being ruled. Yet the same book, the *Politics*, argues that some people are slaves by nature. Centuries later, this idea was used to defend the enslavement of Native Americans.
+**Epicurus (Epicureanism).** Epicurus saw no justice written into nature. For him, justice is an agreement between people not to harm each other, and it can change from place to place. It still matters to the individual: the just person lives with the most peace of mind.
+**Confucius (Confucianism).** Justice begins with the people who lead. A ruler who acts rightly will be followed without needing many orders. When someone wrongs you, answer with justice, not with kindness or revenge. In classical Confucian thought, justice was a personal and public virtue, not a matter of law or equal rights.</t>
+        </is>
+      </c>
+      <c r="V89" s="2" t="inlineStr"/>
+      <c r="W89" s="2" t="inlineStr"/>
+      <c r="X89" s="2" t="inlineStr"/>
+      <c r="Y89" s="2" t="inlineStr">
+        <is>
+          <t>Most agree that justice is about more than rules: it shapes the kind of person you become. They split on where it comes from. For Plato it is part of how things should be; for Epicurus, and later for social contract thinkers like Rousseau, it is something people agree on. Modern debates add new questions the ancients rarely asked, such as how fair inequality can be, as in John Rawls's "veil of ignorance", or whether punishment should aim to repair harm.</t>
+        </is>
+      </c>
+      <c r="Z89" s="2" t="inlineStr"/>
+      <c r="AA89" s="2" t="inlineStr">
         <is>
           <t>- Wikipedia, "Justice": https://en.wikipedia.org/wiki/Justice
 - Wikipedia, "Natural slavery": https://en.wikipedia.org/wiki/Natural_slavery · Stanford Encyclopedia of Philosophy, "Justice": https://plato.stanford.edu/entries/justice/ · "Epicurus": https://plato.stanford.edu/entries/epicurus/ · "Plato's Ethics and Politics in The Republic": https://plato.stanford.edu/entries/plato-ethics-politics/
 - The app's thoughts #71, #84, #85, #98, #127–129, #135, #491, #500, #504, and #617, with their sources</t>
         </is>
       </c>
-      <c r="AB80" s="2" t="inlineStr">
+      <c r="AB89" s="2" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="AC80" s="2" t="inlineStr">
+      <c r="AC89" s="2" t="inlineStr">
         <is>
           <t>Thinker and topic pages pilot</t>
         </is>
       </c>
-      <c r="AD80" s="2" t="inlineStr"/>
+      <c r="AD89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>topic-law-and-rights</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Law and rights</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>**Law and rights** · hand-picked thoughts · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>84,85,127,129,193,491,500,504,590,617,625</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr"/>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>Where do laws get their authority, and what rights do we have?</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr"/>
+      <c r="L90" s="2" t="inlineStr"/>
+      <c r="M90" s="2" t="inlineStr"/>
+      <c r="N90" s="2" t="inlineStr"/>
+      <c r="O90" s="2" t="inlineStr"/>
+      <c r="P90" s="2" t="inlineStr"/>
+      <c r="Q90" s="2" t="inlineStr"/>
+      <c r="R90" s="2" t="inlineStr"/>
+      <c r="S90" s="2" t="inlineStr"/>
+      <c r="T90" s="2" t="inlineStr"/>
+      <c r="U90" s="2" t="inlineStr">
+        <is>
+          <t>**Aristotle (Classical Greek Philosophy).** Is it better to be ruled by the best person or the best laws? Aristotle leaned towards laws, because even good rulers have passions that bend their judgement. The law, he said, is reason unaffected by desire. Without law and justice, the human being is the worst of animals.
+**Confucius (Confucianism).** Confucius trusted example more than rules. To govern means to correct, and a ruler who acts rightly is followed without giving orders. When wronged, repay injury with justice, and kindness with kindness.
+**Epicurus (Epicureanism).** Epicurus saw no justice written into nature. Justice is an agreement between people not to harm each other or be harmed, and it can differ from place to place and time to time.
+**Locke, Rousseau, and Wollstonecraft (Enlightenment Ethics).** Locke argued that all people have natural rights to life, liberty, and property, and that good law does not shrink freedom but protects and enlarges it. Rousseau wanted laws the people make together, and warned that a state is lost once citizens stop caring. Wollstonecraft demanded that rights include women.</t>
+        </is>
+      </c>
+      <c r="V90" s="2" t="inlineStr"/>
+      <c r="W90" s="2" t="inlineStr"/>
+      <c r="X90" s="2" t="inlineStr"/>
+      <c r="Y90" s="2" t="inlineStr">
+        <is>
+          <t>Most of them see good law as a defence against the passions of the powerful; Sa'di put it simply: a tyrant cannot govern, for no one expects the shepherd's duty from the wolf. They split on where law comes from. For Aristotle and Locke, it rests on reason and nature; for Epicurus, on agreement; for Confucius, it matters less than the ruler's character.</t>
+        </is>
+      </c>
+      <c r="Z90" s="2" t="inlineStr"/>
+      <c r="AA90" s="2" t="inlineStr">
+        <is>
+          <t>- Stanford Encyclopedia of Philosophy, "Locke's Political Philosophy": https://plato.stanford.edu/entries/locke-political/ · "Aristotle's Political Theory": https://plato.stanford.edu/entries/aristotle-politics/
+- The app's thoughts listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="AB90" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC90" s="2" t="inlineStr">
+        <is>
+          <t>Society topic pages</t>
+        </is>
+      </c>
+      <c r="AD90" s="2" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>topic-learning-and-knowledge</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Learning and knowledge</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>**Learning and knowledge** · theme: Learning and knowledge · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr"/>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Learning and knowledge</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr"/>
+      <c r="H91" s="2" t="inlineStr"/>
+      <c r="I91" s="2" t="inlineStr"/>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>What is worth knowing, and how do we know that we know it?</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr"/>
+      <c r="L91" s="2" t="inlineStr"/>
+      <c r="M91" s="2" t="inlineStr"/>
+      <c r="N91" s="2" t="inlineStr"/>
+      <c r="O91" s="2" t="inlineStr"/>
+      <c r="P91" s="2" t="inlineStr"/>
+      <c r="Q91" s="2" t="inlineStr"/>
+      <c r="R91" s="2" t="inlineStr"/>
+      <c r="S91" s="2" t="inlineStr"/>
+      <c r="T91" s="2" t="inlineStr"/>
+      <c r="U91" s="2" t="inlineStr">
+        <is>
+          <t>**Socrates and Plato (Classical Greek Philosophy).** Socrates claimed one kind of wisdom: he did not think he knew what he didn't. He questioned people until they saw the limits of their own knowledge, which made him many enemies. For Plato, philosophy begins in wonder, and most of us are like prisoners in a cave, taking shadows for the real thing.
+**Confucius (Confucianism).** Confucius loved learning and said it should never stop. Learning without thinking is wasted, and thinking without learning is dangerous. Real knowledge means saying what you know and admitting what you don't. Anyone can teach you something: copy the good in people, and correct in yourself the bad you see in them.
+**Laozi and Zhuangzi (Taoism).** The Taoists doubted that more knowledge brings more wisdom. Learning adds something every day, but the Way is found by letting go, day by day. Zhuangzi adds that you cannot explain the ocean to a frog in a well: we all see from a narrow place.
+**Hume and Mill (Enlightenment Ethics).** Hume asked for less certainty and more evidence: a wise person matches belief to the evidence. Mill added that you only half know your own view if you have never heard the other side. Even a true belief, never challenged, turns into dead dogma.</t>
+        </is>
+      </c>
+      <c r="V91" s="2" t="inlineStr"/>
+      <c r="W91" s="2" t="inlineStr"/>
+      <c r="X91" s="2" t="inlineStr"/>
+      <c r="Y91" s="2" t="inlineStr">
+        <is>
+          <t>Nearly all of them start with humility: Socrates, Confucius, and Laozi all praise knowing the limits of what you know. They part ways on what to do next. Confucius and Mill say study and argue more; Laozi says empty your mind; Hume says follow the evidence and stay modest about the rest.</t>
+        </is>
+      </c>
+      <c r="Z91" s="2" t="inlineStr"/>
+      <c r="AA91" s="2" t="inlineStr">
+        <is>
+          <t>- Stanford Encyclopedia of Philosophy, "Socrates": https://plato.stanford.edu/entries/socrates/ · "Laozi": https://plato.stanford.edu/entries/laozi/
+- The app's thoughts #96, #97, #104, #162, #167, #175, #418, #420, #429, #470, #471, #480, and #482, with their sources</t>
+        </is>
+      </c>
+      <c r="AB91" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC91" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch A</t>
+        </is>
+      </c>
+      <c r="AD91" s="2" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>topic-love</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Love</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>**Love** · theme: Love · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Love</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr"/>
+      <c r="H92" s="2" t="inlineStr"/>
+      <c r="I92" s="2" t="inlineStr"/>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>What is love, and what does it ask of us?</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr"/>
+      <c r="L92" s="2" t="inlineStr"/>
+      <c r="M92" s="2" t="inlineStr"/>
+      <c r="N92" s="2" t="inlineStr"/>
+      <c r="O92" s="2" t="inlineStr"/>
+      <c r="P92" s="2" t="inlineStr"/>
+      <c r="Q92" s="2" t="inlineStr"/>
+      <c r="R92" s="2" t="inlineStr"/>
+      <c r="S92" s="2" t="inlineStr"/>
+      <c r="T92" s="2" t="inlineStr"/>
+      <c r="U92" s="2" t="inlineStr">
+        <is>
+          <t>**Plato (Classical Greek Philosophy).** In Plato's *Symposium*, guests at a dinner take turns praising love. One tells a myth: humans were once whole beings, cut in two, and love is the desire and pursuit of that lost whole. Then Socrates, quoting his teacher Diotima, describes love as a journey from one beautiful body towards ever purer beauty.
+**Rumi, Hafiz, and Ibn Arabi (Persian and Sufi Poetry).** For the Sufi poets, human love and love of God mirror each other. Love hurts, and the pain is the proof of it. Hafiz admits he thought love would be easy, then found it a hard road. Ibn Arabi wrote that a heart grown in love can take on every form.
+**Tagore and the Dhammapada (Indian Philosophy, Buddhist Philosophy).** Tagore saw love as the way we truly live in the world: when a person loves, giving becomes a joy, like a tree letting go of ripe fruit. The *Dhammapada* gives love a harder task: hatred never ends through hatred, only through love.
+**Dostoevsky (Existential Thought).** Dostoevsky saw how easy it is to love in theory. Love in action, says a monk in *The Brothers Karamazov*, is harsh and dreadful compared with love in dreams. The same monk tells of a doctor who found that the more he loved humanity in general, the less he loved people in particular.</t>
+        </is>
+      </c>
+      <c r="V92" s="2" t="inlineStr"/>
+      <c r="W92" s="2" t="inlineStr"/>
+      <c r="X92" s="2" t="inlineStr"/>
+      <c r="Y92" s="2" t="inlineStr">
+        <is>
+          <t>All of them see love as more than a feeling: it changes the one who loves. They differ on its object. Plato and the Sufi poets point beyond the person towards something higher; Dostoevsky and Montaigne bring it back to one real person, loved, as Montaigne said of his friend, "because it was he, because it was I".</t>
+        </is>
+      </c>
+      <c r="Z92" s="2" t="inlineStr"/>
+      <c r="AA92" s="2" t="inlineStr">
+        <is>
+          <t>- Stanford Encyclopedia of Philosophy, "Plato's Aesthetics": https://plato.stanford.edu/entries/plato-aesthetics/
+- The app's thoughts #106, #219, #221, #280, #308, #378, #389, #559, #567, and #577, with their sources</t>
+        </is>
+      </c>
+      <c r="AB92" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC92" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch B</t>
+        </is>
+      </c>
+      <c r="AD92" s="2" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>topic-mind-and-emotions</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Mind and emotions</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>**Mind and emotions** · theme: Mind and emotions · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>Mind and emotions</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr"/>
+      <c r="H93" s="2" t="inlineStr"/>
+      <c r="I93" s="2" t="inlineStr"/>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>Should we master our feelings, or listen to them?</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr"/>
+      <c r="L93" s="2" t="inlineStr"/>
+      <c r="M93" s="2" t="inlineStr"/>
+      <c r="N93" s="2" t="inlineStr"/>
+      <c r="O93" s="2" t="inlineStr"/>
+      <c r="P93" s="2" t="inlineStr"/>
+      <c r="Q93" s="2" t="inlineStr"/>
+      <c r="R93" s="2" t="inlineStr"/>
+      <c r="S93" s="2" t="inlineStr"/>
+      <c r="T93" s="2" t="inlineStr"/>
+      <c r="U93" s="2" t="inlineStr">
+        <is>
+          <t>**Marcus Aurelius (Stoicism).** For the Stoics, what upsets us is not the event but our judgement about it, and we can learn to judge differently. Marcus Aurelius notes that the mind takes on the colour of its habitual thoughts. The ideal Stoic is free of disturbing passions, though not of all feeling.
+**The Dhammapada (Buddhist Philosophy).** The *Dhammapada* opens with the claim that all we are comes from our thoughts. The mind is flighty and hard to hold, and taming it is the greatest good. Hatred never ends hatred; only love does.
+**Aristotle (Classical Greek Philosophy).** Aristotle did not want feelings gone, but right. Anyone can get angry. The skill is to be angry with the right person, to the right degree, at the right time, and for the right reason. A good character is one that feels the right amount.
+**Spinoza and Hume (Enlightenment Ethics).** Spinoza called being ruled by our emotions a kind of bondage, and said an emotion loses its grip once we understand it clearly. Hume turned the question around: reason on its own moves no one to act, and is, in his words, "the slave of the passions".</t>
+        </is>
+      </c>
+      <c r="V93" s="2" t="inlineStr"/>
+      <c r="W93" s="2" t="inlineStr"/>
+      <c r="X93" s="2" t="inlineStr"/>
+      <c r="Y93" s="2" t="inlineStr">
+        <is>
+          <t>Most of them believe the mind can be trained, and that much suffering comes from how we react. They disagree on the goal. The Stoics and the Buddhist texts aim to calm or uproot troubling passions; Aristotle wants feelings in the right measure; Hume, like Pascal with his "heart" that has its own reasons, gives feeling the leading role.</t>
+        </is>
+      </c>
+      <c r="Z93" s="2" t="inlineStr"/>
+      <c r="AA93" s="2" t="inlineStr">
+        <is>
+          <t>- Stanford Encyclopedia of Philosophy, "Stoicism": https://plato.stanford.edu/entries/stoicism/ · "Aristotle's Ethics": https://plato.stanford.edu/entries/aristotle-ethics/ · "Hume's Moral Philosophy": https://plato.stanford.edu/entries/hume-moral/
+- The app's thoughts #7, #9, #111, #168, #169, #173, #228, #307, #308, and #315, with their sources</t>
+        </is>
+      </c>
+      <c r="AB93" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC93" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch A</t>
+        </is>
+      </c>
+      <c r="AD93" s="2" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>topic-nature-and-the-universe</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Nature and the universe</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>**Nature and the universe** · theme: Nature and the universe · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Nature and the universe</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr"/>
+      <c r="H94" s="2" t="inlineStr"/>
+      <c r="I94" s="2" t="inlineStr"/>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>What is the world made of, and where do we fit in it?</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr"/>
+      <c r="L94" s="2" t="inlineStr"/>
+      <c r="M94" s="2" t="inlineStr"/>
+      <c r="N94" s="2" t="inlineStr"/>
+      <c r="O94" s="2" t="inlineStr"/>
+      <c r="P94" s="2" t="inlineStr"/>
+      <c r="Q94" s="2" t="inlineStr"/>
+      <c r="R94" s="2" t="inlineStr"/>
+      <c r="S94" s="2" t="inlineStr"/>
+      <c r="T94" s="2" t="inlineStr"/>
+      <c r="U94" s="2" t="inlineStr">
+        <is>
+          <t>**Laozi and Zhuangzi (Taoism).** The Tao, the way of nature, cannot be fully named or explained. Its best image is water, which helps everything, takes the lowest place, and still wears away the hardest stone. A person lives well by following that way, not by forcing it.
+**Lucretius and Epicurus (Epicureanism).** For the Epicureans, everything is made of atoms moving in empty space; worlds form by chance, without any need for gods. Lucretius wrote that fear comes from not knowing the causes of things. Understanding nature, he said, is the cure for that fear.
+**Marcus Aurelius and Epictetus (Stoicism).** The Stoics saw the opposite: one living whole, shaped by reason, in which every part is connected. Marcus Aurelius told himself to see the universe as a single being with one substance and one soul. Epictetus reminded his students how small a part of it each of us is.
+**Kant and Pascal (Enlightenment Ethics, Existential Thought).** Two things filled Kant with ever-growing awe: the starry heavens above and the moral law within. Pascal saw human beings as reeds, the weakest thing in nature, but reeds that think, and our greatness lies in that thought.</t>
+        </is>
+      </c>
+      <c r="V94" s="2" t="inlineStr"/>
+      <c r="W94" s="2" t="inlineStr"/>
+      <c r="X94" s="2" t="inlineStr"/>
+      <c r="Y94" s="2" t="inlineStr">
+        <is>
+          <t>All of them say that understanding nature changes how we live in it. They split on whether it has a purpose. The Stoics see a rational order; the Epicureans see atoms and chance; the Taoists see a way that cannot be put into words. The Japanese writers add something simpler: notice it, from the dawn to the flowers.</t>
+        </is>
+      </c>
+      <c r="Z94" s="2" t="inlineStr"/>
+      <c r="AA94" s="2" t="inlineStr">
+        <is>
+          <t>- Stanford Encyclopedia of Philosophy, "Lucretius": https://plato.stanford.edu/entries/lucretius/ · "Stoicism": https://plato.stanford.edu/entries/stoicism/
+- The app's thoughts #37, #44, #87, #89, #152, #226, #410, #422, #441, #543, and #553, with their sources</t>
+        </is>
+      </c>
+      <c r="AB94" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC94" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch B</t>
+        </is>
+      </c>
+      <c r="AD94" s="2" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>topic-purpose-and-meaning</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Purpose and meaning</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>**Purpose and meaning** · theme: Purpose and meaning · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Purpose and meaning</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr"/>
+      <c r="H95" s="2" t="inlineStr"/>
+      <c r="I95" s="2" t="inlineStr"/>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>What is a life for?</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr"/>
+      <c r="L95" s="2" t="inlineStr"/>
+      <c r="M95" s="2" t="inlineStr"/>
+      <c r="N95" s="2" t="inlineStr"/>
+      <c r="O95" s="2" t="inlineStr"/>
+      <c r="P95" s="2" t="inlineStr"/>
+      <c r="Q95" s="2" t="inlineStr"/>
+      <c r="R95" s="2" t="inlineStr"/>
+      <c r="S95" s="2" t="inlineStr"/>
+      <c r="T95" s="2" t="inlineStr"/>
+      <c r="U95" s="2" t="inlineStr">
+        <is>
+          <t>**Aristotle (Classical Greek Philosophy).** Aristotle noticed that everything we do aims at some good, and those goods point to a final one: happiness, the thing we want for its own sake. For him, the question of meaning had an answer: a life of reason and virtue, lived well.
+**Tolstoy and William James (Existential Thought).** Tolstoy had fame, family, and wealth when his life "came to a standstill": he could no longer see what any of it was for. William James answered the same fear in a lecture called "Is Life Worth Living?". We live fully, he said, only by risking ourselves on what we believe.
+**Mill (Enlightenment Ethics).** At twenty, Mill asked himself whether reaching all his goals would make him happy, and an honest voice said no. He came out of the crisis with a lesson: happiness comes to those who aim at something other than their own happiness.
+**George Eliot, Dickinson, and Tagore (Humanists and Essayists, Indian Philosophy).** Many find meaning in what we do for others. "What do we live for," asks a character in *Middlemarch*, "if it is not to make life less difficult to each other?" Dickinson would not live in vain if she could stop one heart from breaking, and Tagore says we earn our life by giving it.</t>
+        </is>
+      </c>
+      <c r="V95" s="2" t="inlineStr"/>
+      <c r="W95" s="2" t="inlineStr"/>
+      <c r="X95" s="2" t="inlineStr"/>
+      <c r="Y95" s="2" t="inlineStr">
+        <is>
+          <t>Most of them say meaning comes from something larger than the self, whether virtue, a cause, or other people. They differ on whether it is given or made. Aristotle finds it in human nature; Nietzsche says you must become what you are; Zhuangzi gently mocks the whole idea, praising a useless tree that lives long because nobody wants it.</t>
+        </is>
+      </c>
+      <c r="Z95" s="2" t="inlineStr"/>
+      <c r="AA95" s="2" t="inlineStr">
+        <is>
+          <t>- The app's thoughts #116, #144, #163, #166, #214, #240, #243, #288, #296, #385, and #434, with their sources</t>
+        </is>
+      </c>
+      <c r="AB95" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC95" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch B</t>
+        </is>
+      </c>
+      <c r="AD95" s="2" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>topic-self-knowledge</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Self-knowledge</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>**Self-knowledge** · theme: Self-knowledge · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Self-knowledge</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr"/>
+      <c r="H96" s="2" t="inlineStr"/>
+      <c r="I96" s="2" t="inlineStr"/>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>Who are you, really, and can you ever know?</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr"/>
+      <c r="M96" s="2" t="inlineStr"/>
+      <c r="N96" s="2" t="inlineStr"/>
+      <c r="O96" s="2" t="inlineStr"/>
+      <c r="P96" s="2" t="inlineStr"/>
+      <c r="Q96" s="2" t="inlineStr"/>
+      <c r="R96" s="2" t="inlineStr"/>
+      <c r="S96" s="2" t="inlineStr"/>
+      <c r="T96" s="2" t="inlineStr"/>
+      <c r="U96" s="2" t="inlineStr">
+        <is>
+          <t>**Socrates (Classical Greek Philosophy).** At his trial, Socrates said the unexamined life is not worth living. For him, questioning yourself and others was not a hobby but a duty, worth dying for.
+**The Upanishads and the Buddhist texts (Indian Philosophy, Buddhist Philosophy).** The Upanishads look for a deep, lasting Self behind body and mind, and find it one with the Self in all beings. Buddhism turns this around. In *The Questions of King Milinda*, a chariot is just a name for its parts working together, and so is a person: there is no fixed self to find.
+**Confucius (Confucianism).** For Confucius, self-knowledge is daily practice. One of his students examined himself every day on three points: had he been loyal, been true to his friends, and practised what he was taught? The superior man looks for the cause of things in himself; the petty man looks for it in others.
+**Montaigne and La Rochefoucauld (Humanists and Essayists).** Montaigne made himself the subject of his *Essays*, because each person carries the whole human condition. La Rochefoucauld was less hopeful: we are so used to wearing masks for others that in the end we are disguised to ourselves.</t>
+        </is>
+      </c>
+      <c r="V96" s="2" t="inlineStr"/>
+      <c r="W96" s="2" t="inlineStr"/>
+      <c r="X96" s="2" t="inlineStr"/>
+      <c r="Y96" s="2" t="inlineStr">
+        <is>
+          <t>They all say the work begins inside, not in other people's opinions. They differ on what you find there: a lasting Self (the Upanishads), no fixed self at all (Buddhism), a self you still have to create (Nietzsche's "become what you are"), or a mirror of everyone (Montaigne).</t>
+        </is>
+      </c>
+      <c r="Z96" s="2" t="inlineStr"/>
+      <c r="AA96" s="2" t="inlineStr">
+        <is>
+          <t>- Stanford Encyclopedia of Philosophy, "Socrates": https://plato.stanford.edu/entries/socrates/
+- The app's thoughts #95, #214, #273, #283, #355, #364, #366, #493, and #513, with their sources</t>
+        </is>
+      </c>
+      <c r="AB96" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC96" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch A</t>
+        </is>
+      </c>
+      <c r="AD96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>topic-solitude-and-stillness</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Solitude and stillness</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>**Solitude and stillness** · theme: Solitude and stillness · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Solitude and stillness</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr"/>
+      <c r="H97" s="2" t="inlineStr"/>
+      <c r="I97" s="2" t="inlineStr"/>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>Why is it so hard to sit still, and what do we find when we do?</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr"/>
+      <c r="L97" s="2" t="inlineStr"/>
+      <c r="M97" s="2" t="inlineStr"/>
+      <c r="N97" s="2" t="inlineStr"/>
+      <c r="O97" s="2" t="inlineStr"/>
+      <c r="P97" s="2" t="inlineStr"/>
+      <c r="Q97" s="2" t="inlineStr"/>
+      <c r="R97" s="2" t="inlineStr"/>
+      <c r="S97" s="2" t="inlineStr"/>
+      <c r="T97" s="2" t="inlineStr"/>
+      <c r="U97" s="2" t="inlineStr">
+        <is>
+          <t>**Pascal (Existential Thought).** Pascal thought all human misfortune comes from one thing: we cannot stay quietly in a room. We chase distraction to avoid thinking about ourselves, and that distraction is itself our greatest misery.
+**Marcus Aurelius (Stoicism).** While ruling an empire, Marcus longed for a house in the country or by the sea, as rich Romans had. Then he reminded himself that he could retreat into his own mind whenever he chose, and that there is no quieter place.
+**Laozi and Zhuangzi (Taoism).** Muddy water, says the *Tao Te Ching*, becomes clear if you let it be still. Zhuangzi says the wise use the mind like a mirror: it grasps nothing and refuses nothing, and reflects what comes without holding on.
+**Kenkō and Chōmei (Japanese Aesthetics).** The Japanese recluses praised a quiet life away from the crowd. Kenkō asked how anyone could find leisure tiresome: free from cares, it is good simply to be alone. From his small hut, Chōmei watched the moon at his window and thought of people of old.</t>
+        </is>
+      </c>
+      <c r="V97" s="2" t="inlineStr"/>
+      <c r="W97" s="2" t="inlineStr"/>
+      <c r="X97" s="2" t="inlineStr"/>
+      <c r="Y97" s="2" t="inlineStr">
+        <is>
+          <t>All of them see stillness as the place where the mind clears. They differ on how alone to be. Schopenhauer and Nietzsche praise solitude itself, and the *Dhammapada* says it is better to travel alone than with a fool. For Marcus, though, the retreat is inward and can be taken anywhere, even in the middle of public life.</t>
+        </is>
+      </c>
+      <c r="Z97" s="2" t="inlineStr"/>
+      <c r="AA97" s="2" t="inlineStr">
+        <is>
+          <t>- The app's thoughts #3, #215, #225, #229, #230, #354, #417, #438, #522, and #541, with their sources</t>
+        </is>
+      </c>
+      <c r="AB97" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC97" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch B</t>
+        </is>
+      </c>
+      <c r="AD97" s="2" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>topic-suffering-and-resilience</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Suffering and resilience</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>**Suffering and resilience** · theme: Suffering and resilience · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Suffering and resilience</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr"/>
+      <c r="H98" s="2" t="inlineStr"/>
+      <c r="I98" s="2" t="inlineStr"/>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>What do we do with pain we cannot avoid?</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr"/>
+      <c r="L98" s="2" t="inlineStr"/>
+      <c r="M98" s="2" t="inlineStr"/>
+      <c r="N98" s="2" t="inlineStr"/>
+      <c r="O98" s="2" t="inlineStr"/>
+      <c r="P98" s="2" t="inlineStr"/>
+      <c r="Q98" s="2" t="inlineStr"/>
+      <c r="R98" s="2" t="inlineStr"/>
+      <c r="S98" s="2" t="inlineStr"/>
+      <c r="T98" s="2" t="inlineStr"/>
+      <c r="U98" s="2" t="inlineStr">
+        <is>
+          <t>**Marcus Aurelius, Epictetus, and Boethius (Stoicism).** Marcus Aurelius asked to be like a headland that the waves keep breaking on, while it stands firm. Epictetus advised wishing for things to happen as they do, not as we would like. In prison, Boethius wrote that nothing is wretched unless we think it so.
+**Rumi and Hafiz (Persian and Sufi Poetry).** The Sufi poets see pain as part of the way. Rumi calls it a treasure that holds mercies, and the *Masnavi* opens with a reed flute crying for the reed bed it was cut from. Hafiz says no one reaches joy without passing through hardship.
+**Nietzsche and Dostoevsky (Existential Thought).** Nietzsche's answer was *amor fati*, love of fate: wanting nothing to be different, the hard parts included. Dostoevsky went further, calling suffering the origin of consciousness itself.
+**Weil and Mill (Existential Thought, Enlightenment Ethics).** Others look outward. Simone Weil said those who suffer need, above all, people able to pay them attention. And Mill believed most of the great causes of suffering can be reduced by human care and effort.</t>
+        </is>
+      </c>
+      <c r="V98" s="2" t="inlineStr"/>
+      <c r="W98" s="2" t="inlineStr"/>
+      <c r="X98" s="2" t="inlineStr"/>
+      <c r="Y98" s="2" t="inlineStr">
+        <is>
+          <t>Many of them say suffering can teach and deepen us, as Vivekananda put it: misery is sometimes a greater teacher than happiness. They differ on where the answer lies. The Stoics look to our own judgement, the Sufi poets to love and longing, Weil to other people, and Mill to changing the world itself.</t>
+        </is>
+      </c>
+      <c r="Z98" s="2" t="inlineStr"/>
+      <c r="AA98" s="2" t="inlineStr">
+        <is>
+          <t>- The app's thoughts #6, #17, #28, #199, #213, #236, #248, #380, #555, #570, and #596, with their sources</t>
+        </is>
+      </c>
+      <c r="AB98" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC98" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch B</t>
+        </is>
+      </c>
+      <c r="AD98" s="2" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>topic-time-and-the-present</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Time and the present</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>**Time and the present** · theme: Time and the present · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>Time and the present</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr"/>
+      <c r="H99" s="2" t="inlineStr"/>
+      <c r="I99" s="2" t="inlineStr"/>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>Is life short, or do we waste it?</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr"/>
+      <c r="L99" s="2" t="inlineStr"/>
+      <c r="M99" s="2" t="inlineStr"/>
+      <c r="N99" s="2" t="inlineStr"/>
+      <c r="O99" s="2" t="inlineStr"/>
+      <c r="P99" s="2" t="inlineStr"/>
+      <c r="Q99" s="2" t="inlineStr"/>
+      <c r="R99" s="2" t="inlineStr"/>
+      <c r="S99" s="2" t="inlineStr"/>
+      <c r="T99" s="2" t="inlineStr"/>
+      <c r="U99" s="2" t="inlineStr">
+        <is>
+          <t>**Seneca (Stoicism).** Seneca argued that life is not short; we make it short by wasting it. How late, he said, to begin living just when we must leave. Epictetus added that he wanted to be present like the hour, and to pass like the hour.
+**Epicurus (Epicureanism).** Epicurus warned against putting off joy for a tomorrow we do not control. The future is neither fully ours nor fully out of our hands. And remembering the good days we have had is part of a happy life.
+**Omar Khayyam and Hafiz (Persian and Sufi Poetry).** The Persian poets feel time slipping past. Khayyam's "Moving Finger" writes and moves on, and nothing can make it go back. Their answer is to make the most of the days we have.
+**Kenkō and Pascal (Japanese Aesthetics, Existential Thought).** Kenkō noted that the seasons come in order, but death comes when it likes, so we should not put off what matters. Pascal saw the same habit from another side: we never live, but only hope to live.</t>
+        </is>
+      </c>
+      <c r="V99" s="2" t="inlineStr"/>
+      <c r="W99" s="2" t="inlineStr"/>
+      <c r="X99" s="2" t="inlineStr"/>
+      <c r="Y99" s="2" t="inlineStr">
+        <is>
+          <t>All of them say the present is the only time we truly have. They differ on what to fill it with: pleasure and wine for Khayyam, wisdom and duty for Seneca, quiet attention for Kenkō. Montaigne sums up the common ground: life is measured by its use, not its length.</t>
+        </is>
+      </c>
+      <c r="Z99" s="2" t="inlineStr"/>
+      <c r="AA99" s="2" t="inlineStr">
+        <is>
+          <t>- The app's thoughts #24, #26, #43, #63, #77, #79, #227, #278, #520, #579, and #583, with their sources</t>
+        </is>
+      </c>
+      <c r="AB99" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC99" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch A</t>
+        </is>
+      </c>
+      <c r="AD99" s="2" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>topic-tolerance</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Tolerance</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>**Tolerance** · hand-picked thoughts · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr"/>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>160,201,550,577,613,614,624</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr"/>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>How do we live with people who believe differently?</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="inlineStr"/>
+      <c r="M100" s="2" t="inlineStr"/>
+      <c r="N100" s="2" t="inlineStr"/>
+      <c r="O100" s="2" t="inlineStr"/>
+      <c r="P100" s="2" t="inlineStr"/>
+      <c r="Q100" s="2" t="inlineStr"/>
+      <c r="R100" s="2" t="inlineStr"/>
+      <c r="S100" s="2" t="inlineStr"/>
+      <c r="T100" s="2" t="inlineStr"/>
+      <c r="U100" s="2" t="inlineStr">
+        <is>
+          <t>**Locke (Enlightenment Ethics).** In *A Letter Concerning Toleration* (1689), Locke argued that faith cannot be forced, so the state should not try. Churches are voluntary groups, and religion is a matter for each person. But his tolerance had limits: he refused it to atheists, whose promises he thought could not be trusted, and to churches whose members owed loyalty to a foreign ruler.
+**Voltaire (Enlightenment Ethics).** After a Protestant merchant, Jean Calas, was executed in Toulouse in 1762 on a false charge, Voltaire wrote his *Treatise on Tolerance*. In his *Philosophical Dictionary* he calls tolerance the mark of our humanity: we are all made of weakness and error, so let us forgive each other's foolishness. Prejudice, he adds, is an opinion without judgement, taught to children before they can think.
+**Mill (Enlightenment Ethics).** Mill moved the question from religion to every kind of opinion. If all of humanity but one person agreed, they would have no more right to silence that person than the one would have to silence them. Silencing a view, he said, assumes we cannot be wrong.
+**Ibn Arabi and Okakura (Persian and Sufi Poetry, Japanese Aesthetics).** Ibn Arabi wrote of a heart that can take on every form: a monastery, a temple, a place of pilgrimage. Okakura, writing in English for Western readers, said East and West had grown along different lines, with no reason why one should not complete the other.</t>
+        </is>
+      </c>
+      <c r="V100" s="2" t="inlineStr"/>
+      <c r="W100" s="2" t="inlineStr"/>
+      <c r="X100" s="2" t="inlineStr"/>
+      <c r="Y100" s="2" t="inlineStr">
+        <is>
+          <t>All of them see that forcing belief does not work and that our own views may be wrong. They disagree on the limits. Locke still excluded some groups; Voltaire mostly had religious violence in mind; Mill defended almost any opinion, short of harm to others.</t>
+        </is>
+      </c>
+      <c r="Z100" s="2" t="inlineStr"/>
+      <c r="AA100" s="2" t="inlineStr">
+        <is>
+          <t>- Stanford Encyclopedia of Philosophy, "Toleration": https://plato.stanford.edu/entries/toleration/
+- Wikipedia, "A Letter Concerning Toleration": https://en.wikipedia.org/wiki/A_Letter_Concerning_Toleration · "Treatise on Tolerance": https://en.wikipedia.org/wiki/Treatise_on_Tolerance
+- The app's thoughts listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="AB100" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC100" s="2" t="inlineStr">
+        <is>
+          <t>Society topic pages</t>
+        </is>
+      </c>
+      <c r="AD100" s="2" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>topic-war-and-peace</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>War and peace</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>**War and peace** · hand-picked thoughts · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr"/>
+      <c r="F101" s="2" t="inlineStr"/>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>310,330,452,592,616,623</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr"/>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>Can war ever be right, and what makes peace last?</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr"/>
+      <c r="L101" s="2" t="inlineStr"/>
+      <c r="M101" s="2" t="inlineStr"/>
+      <c r="N101" s="2" t="inlineStr"/>
+      <c r="O101" s="2" t="inlineStr"/>
+      <c r="P101" s="2" t="inlineStr"/>
+      <c r="Q101" s="2" t="inlineStr"/>
+      <c r="R101" s="2" t="inlineStr"/>
+      <c r="S101" s="2" t="inlineStr"/>
+      <c r="T101" s="2" t="inlineStr"/>
+      <c r="U101" s="2" t="inlineStr">
+        <is>
+          <t>**Laozi and the Dhammapada (Taoism, Buddhist Philosophy).** The *Tao Te Ching* says the most skilled warrior shows no warlike look and never gives way to rage. The *Dhammapada* sees what victory costs: it breeds hatred, because the loser is unhappy. And the greatest victory is over yourself, not over a thousand armies.
+**The Bhagavad Gita (Indian Philosophy).** The *Gita* is set on a battlefield. Prince Arjuna sees relatives, friends, and teachers in the enemy ranks, drops his bow, and refuses to fight. Krishna urges him to do his duty as a warrior. Yet Gandhi learned the last verses of its second chapter by heart and kept them as a companion in his non-violent movement.
+**Hobbes and Kant (Enlightenment Ethics).** Hobbes, who lived through civil war, described life without government as a war of all against all. Peace, for him, needs a strong ruler; a commonwealth, he wrote, is the mother of peace. Kant hoped for more: in *Towards Perpetual Peace* (1795) he proposed republics joined in a union of states.
+**Voltaire and Tolstoy (Enlightenment Ethics, Existential Thought).** Voltaire noted a sad truth: wishing your country to be great usually means wishing harm on your neighbours. Tolstoy went furthest: read literally, he said, the Sermon on the Mount forbids resisting evil by force. His ideas on non-violence deeply impressed Gandhi.</t>
+        </is>
+      </c>
+      <c r="V101" s="2" t="inlineStr"/>
+      <c r="W101" s="2" t="inlineStr"/>
+      <c r="X101" s="2" t="inlineStr"/>
+      <c r="Y101" s="2" t="inlineStr">
+        <is>
+          <t>None of them see war as glorious in itself. They split on whether it can be justified. The *Gita* accepts a just duty to fight, and Hobbes and Kant seek peace through political order; Tolstoy rejects violence altogether. Sa'di adds a quieter thought: a falsehood that brings peace can be better than a truth that stirs up harm.</t>
+        </is>
+      </c>
+      <c r="Z101" s="2" t="inlineStr"/>
+      <c r="AA101" s="2" t="inlineStr">
+        <is>
+          <t>- Wikipedia, "Bhagavad Gita": https://en.wikipedia.org/wiki/Bhagavad_Gita · "The Kingdom of God Is Within You": https://en.wikipedia.org/wiki/The_Kingdom_of_God_Is_Within_You
+- Stanford Encyclopedia of Philosophy, "Hobbes's Moral and Political Philosophy": https://plato.stanford.edu/entries/hobbes-moral/ · "Kant's Social and Political Philosophy": https://plato.stanford.edu/entries/kant-social-political/
+- The app's thoughts listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="AB101" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC101" s="2" t="inlineStr">
+        <is>
+          <t>Society topic pages</t>
+        </is>
+      </c>
+      <c r="AD101" s="2" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>topic-work-and-action</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Work and action</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>**Work and action** · theme: Work and action · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr"/>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Work and action</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr"/>
+      <c r="H102" s="2" t="inlineStr"/>
+      <c r="I102" s="2" t="inlineStr"/>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>How should we act, and what should we expect from it?</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr"/>
+      <c r="L102" s="2" t="inlineStr"/>
+      <c r="M102" s="2" t="inlineStr"/>
+      <c r="N102" s="2" t="inlineStr"/>
+      <c r="O102" s="2" t="inlineStr"/>
+      <c r="P102" s="2" t="inlineStr"/>
+      <c r="Q102" s="2" t="inlineStr"/>
+      <c r="R102" s="2" t="inlineStr"/>
+      <c r="S102" s="2" t="inlineStr"/>
+      <c r="T102" s="2" t="inlineStr"/>
+      <c r="U102" s="2" t="inlineStr">
+        <is>
+          <t>**The Bhagavad Gita and Vivekananda (Indian Philosophy).** In the *Gita*, Krishna tells Arjuna that his business is with the action alone, never with its fruits. It is better to do your own task imperfectly than someone else's well. Vivekananda put it simply: work without stopping, but without attachment.
+**Marcus Aurelius (Stoicism).** Even an emperor found it hard to get up in the morning. His reminder to himself: I am rising to do the work of a human being. He also told himself to stop talking about what a good man should be, and simply be one.
+**Laozi and Zhuangzi (Taoism).** The Taoists value action that does not force. Governing a great state, says the *Tao Te Ching*, is like cooking small fish: stir too much and they fall apart. Zhuangzi's cook works with the grain of things, and his knife stays sharp for nineteen years.
+**Confucius and Voltaire (Confucianism, Enlightenment Ethics).** Confucius praised the person who acts first and speaks afterwards. At the end of Voltaire's *Candide*, after war, shipwreck, and earthquake, the hero stops arguing about whether all is for the best. "We must cultivate our garden."</t>
+        </is>
+      </c>
+      <c r="V102" s="2" t="inlineStr"/>
+      <c r="W102" s="2" t="inlineStr"/>
+      <c r="X102" s="2" t="inlineStr"/>
+      <c r="Y102" s="2" t="inlineStr">
+        <is>
+          <t>All of them trust deeds over words. They differ on effort and reward. The *Gita* and the Stoics speak of duty done well whatever the result; the Taoists warn against forcing things; Voltaire suggests that useful work close to home may be the best answer to questions we cannot solve.</t>
+        </is>
+      </c>
+      <c r="Z102" s="2" t="inlineStr"/>
+      <c r="AA102" s="2" t="inlineStr">
+        <is>
+          <t>- The app's thoughts #10, #12, #360, #368, #381, #432, #449, #472, and #611, with their sources</t>
+        </is>
+      </c>
+      <c r="AB102" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC102" s="2" t="inlineStr">
+        <is>
+          <t>Theme pages, batch B</t>
+        </is>
+      </c>
+      <c r="AD102" s="2" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>topic-work-and-wealth</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Work and wealth</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>**Work and wealth** · hand-picked thoughts · [n] thoughts so far</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr"/>
+      <c r="F103" s="2" t="inlineStr"/>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>12,61,184,252,406,479,489,521,575,622</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr"/>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>How much is enough, and what is work for?</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr"/>
+      <c r="L103" s="2" t="inlineStr"/>
+      <c r="M103" s="2" t="inlineStr"/>
+      <c r="N103" s="2" t="inlineStr"/>
+      <c r="O103" s="2" t="inlineStr"/>
+      <c r="P103" s="2" t="inlineStr"/>
+      <c r="Q103" s="2" t="inlineStr"/>
+      <c r="R103" s="2" t="inlineStr"/>
+      <c r="S103" s="2" t="inlineStr"/>
+      <c r="T103" s="2" t="inlineStr"/>
+      <c r="U103" s="2" t="inlineStr">
+        <is>
+          <t>**Epicurus and Marcus Aurelius (Epicureanism, Stoicism).** Epicurus said nature's wealth is limited and easy to get, while the wealth of empty wishes has no end. Marcus Aurelius, emperor of Rome, reminded himself each morning that he was rising to do the work of a human being.
+**Confucius and Sa'di (Confucianism, Persian and Sufi Poetry).** Confucius could find joy with coarse rice and water, and called riches gained by wrongdoing a floating cloud. Being poor without complaining is hard, he said; being rich without pride is easy. Sa'di advised anyone who wants riches to ask for contentment instead.
+**Adam Smith and Rousseau (Enlightenment Ethics).** Adam Smith argued in *The Wealth of Nations* that wealth grows through free exchange and the division of labour, as if guided by an "invisible hand". Yet his first book began with sympathy: however selfish we are, we care about others' happiness. Rousseau saw a darker side: the first person who fenced off land, said "This is mine", and found people simple enough to believe it, opened the way to crimes, wars, and misery.
+**Vivekananda and Schopenhauer (Indian Philosophy, Existential Thought).** Vivekananda taught that the best work is done for no reward, neither money nor fame. Schopenhauer compared riches to sea water: the more you drink, the thirstier you get.</t>
+        </is>
+      </c>
+      <c r="V103" s="2" t="inlineStr"/>
+      <c r="W103" s="2" t="inlineStr"/>
+      <c r="X103" s="2" t="inlineStr"/>
+      <c r="Y103" s="2" t="inlineStr">
+        <is>
+          <t>Most of them warn that wealth beyond need rarely brings peace. They differ on what wealth does for society. Smith saw trade and work as the way whole nations grow richer; Rousseau saw property as the root of inequality; the Stoics and the *Gita* tradition care less about the wealth than about the spirit in which we work.</t>
+        </is>
+      </c>
+      <c r="Z103" s="2" t="inlineStr"/>
+      <c r="AA103" s="2" t="inlineStr">
+        <is>
+          <t>- Wikipedia, "The Wealth of Nations": https://en.wikipedia.org/wiki/The_Wealth_of_Nations · Stanford Encyclopedia of Philosophy, "Adam Smith's Moral and Political Philosophy": https://plato.stanford.edu/entries/smith-moral-political/
+- The app's thoughts listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="AB103" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="AC103" s="2" t="inlineStr">
+        <is>
+          <t>Society topic pages</t>
+        </is>
+      </c>
+      <c r="AD103" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7714,7 +9569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C253"/>
+  <dimension ref="A1:C304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -11363,377 +13218,1152 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>topic-democracy</t>
+          <t>topic-beauty-and-art</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Wikipedia, "Athenian democracy"</t>
+          <t>Stanford Encyclopedia of Philosophy, "Hume's Aesthetics"</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Athenian_democracy</t>
+          <t>https://plato.stanford.edu/entries/hume-aesthetics/</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>topic-democracy</t>
+          <t>topic-beauty-and-art</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Stanford Encyclopedia of Philosophy, "Aristotle's Political Theory"</t>
-        </is>
-      </c>
-      <c r="C232" t="inlineStr">
-        <is>
-          <t>https://plato.stanford.edu/entries/aristotle-politics/</t>
-        </is>
-      </c>
+          <t>The app's thoughts #177, #188, #259, #264, #421, #525, #533, and #534, with their sources</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>topic-democracy</t>
+          <t>topic-change-and-impermanence</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>"Plato's Ethics and Politics in The Republic"</t>
-        </is>
-      </c>
-      <c r="C233" t="inlineStr">
-        <is>
-          <t>https://plato.stanford.edu/entries/plato-ethics-politics/</t>
-        </is>
-      </c>
+          <t>The app's thoughts #18, #33, #88, #121, #209, #345, #515, #517, and #529, with their sources</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>topic-democracy</t>
+          <t>topic-character-and-virtue</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Plato, Republic, Book VI (Jowett translation, Project Gutenberg)</t>
+          <t>Stanford Encyclopedia of Philosophy, "Virtue Ethics"</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>https://www.gutenberg.org/ebooks/1497</t>
+          <t>https://plato.stanford.edu/entries/ethics-virtue/</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>topic-democracy</t>
+          <t>topic-character-and-virtue</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Wikipedia, "Tyranny of the majority"</t>
+          <t>Stanford Encyclopedia of Philosophy, "Kant's Moral Philosophy"</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Tyranny_of_the_majority</t>
+          <t>https://plato.stanford.edu/entries/kant-moral/</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>topic-democracy</t>
+          <t>topic-character-and-virtue</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>The app's thoughts listed above, with their sources</t>
-        </is>
-      </c>
-      <c r="C236" t="inlineStr"/>
+          <t>"Confucius"</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/confucius/</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>topic-freedom</t>
+          <t>topic-character-and-virtue</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Stanford Encyclopedia of Philosophy, "Positive and Negative Liberty"</t>
-        </is>
-      </c>
-      <c r="C237" t="inlineStr">
-        <is>
-          <t>https://plato.stanford.edu/entries/liberty-positive-negative/</t>
-        </is>
-      </c>
+          <t>The app's thoughts #109, #113, #119, #154, #155, #208, #328, #333, #339, #357, #475, #487, #492, #495, and #504, with their sources</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>topic-freedom</t>
+          <t>topic-death-and-mortality</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>John Stuart Mill, *On Liberty* (1859), chapter I (Project Gutenberg)</t>
-        </is>
-      </c>
-      <c r="C238" t="inlineStr">
-        <is>
-          <t>https://www.gutenberg.org/ebooks/34901</t>
-        </is>
-      </c>
+          <t>The app's thoughts #4, #59, #73, #75, #170, #277, #387, #437, #520, #582, and #583, with their sources</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>topic-freedom</t>
+          <t>topic-democracy</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Wikipedia, "Negative liberty"</t>
+          <t>Wikipedia, "Athenian democracy"</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Negative_liberty</t>
+          <t>https://en.wikipedia.org/wiki/Athenian_democracy</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>topic-freedom</t>
+          <t>topic-democracy</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Stanford Encyclopedia of Philosophy, 2014 version of the same entry (on the Stoics)</t>
+          <t>Stanford Encyclopedia of Philosophy, "Aristotle's Political Theory"</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>https://plato.stanford.edu/archives/sum2014/entries/liberty-positive-negative/</t>
+          <t>https://plato.stanford.edu/entries/aristotle-politics/</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>topic-freedom</t>
+          <t>topic-democracy</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>The app's thoughts #15, #42, #168, #197, #198, and the others listed above, with their sources</t>
-        </is>
-      </c>
-      <c r="C241" t="inlineStr"/>
+          <t>"Plato's Ethics and Politics in The Republic"</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/plato-ethics-politics/</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>topic-friendship</t>
+          <t>topic-democracy</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Stanford Encyclopedia of Philosophy, "Friendship"</t>
+          <t>Plato, Republic, Book VI (Jowett translation, Project Gutenberg)</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>https://plato.stanford.edu/entries/friendship/</t>
+          <t>https://www.gutenberg.org/ebooks/1497</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>topic-friendship</t>
+          <t>topic-democracy</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Wikipedia, "Epicurus"</t>
+          <t>Wikipedia, "Tyranny of the majority"</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Epicurus</t>
+          <t>https://en.wikipedia.org/wiki/Tyranny_of_the_majority</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>topic-friendship</t>
+          <t>topic-democracy</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Cambridge University Library, "Of friendship" (Montaigne exhibition)</t>
-        </is>
-      </c>
-      <c r="C244" t="inlineStr">
-        <is>
-          <t>https://wwwe.lib.cam.ac.uk/CUL/exhibitions/Montaigne/c3.html</t>
-        </is>
-      </c>
+          <t>The app's thoughts listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>topic-friendship</t>
+          <t>topic-desire-and-simplicity</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Montaigne, "Of Friendship", Cotton translation (HyperEssays)</t>
-        </is>
-      </c>
-      <c r="C245" t="inlineStr">
-        <is>
-          <t>https://hyperessays.net/essays/on-friendship/</t>
-        </is>
-      </c>
+          <t>The app's thoughts #5, #25, #41, #61, #72, #182, #194, #254, #267, #268, #353, #368, #370, and #419, with their sources</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>topic-friendship</t>
+          <t>topic-ego-pride-and-humility</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Wikipedia, "Michel de Montaigne"</t>
-        </is>
-      </c>
-      <c r="C246" t="inlineStr">
-        <is>
-          <t>https://en.wikipedia.org/wiki/Michel_de_Montaigne</t>
-        </is>
-      </c>
+          <t>The app's thoughts #23, #44, #290, #301, #410, #411, #415, #468, #483, and #490, with their sources</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>topic-friendship</t>
+          <t>topic-equality</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>The app's thoughts #58, #112, #115, #117, #211, #280, #502, and #503, with their sources</t>
-        </is>
-      </c>
-      <c r="C247" t="inlineStr"/>
+          <t>Stanford Encyclopedia of Philosophy, "Equality"</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/equality/</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>topic-justice</t>
+          <t>topic-equality</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Wikipedia, "Justice"</t>
+          <t>Wikipedia, "Natural slavery"</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Justice</t>
+          <t>https://en.wikipedia.org/wiki/Natural_slavery</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>topic-justice</t>
+          <t>topic-equality</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Wikipedia, "Natural slavery"</t>
+          <t>Stanford Encyclopedia of Philosophy, "Jean Jacques Rousseau"</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Natural_slavery</t>
+          <t>https://plato.stanford.edu/entries/rousseau/</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>topic-justice</t>
+          <t>topic-equality</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Stanford Encyclopedia of Philosophy, "Justice"</t>
-        </is>
-      </c>
-      <c r="C250" t="inlineStr">
-        <is>
-          <t>https://plato.stanford.edu/entries/justice/</t>
-        </is>
-      </c>
+          <t>The app's thoughts listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>topic-justice</t>
+          <t>topic-freedom</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>"Epicurus"</t>
+          <t>Stanford Encyclopedia of Philosophy, "Positive and Negative Liberty"</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>https://plato.stanford.edu/entries/epicurus/</t>
+          <t>https://plato.stanford.edu/entries/liberty-positive-negative/</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>topic-justice</t>
+          <t>topic-freedom</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>"Plato's Ethics and Politics in The Republic"</t>
+          <t>John Stuart Mill, *On Liberty* (1859), chapter I (Project Gutenberg)</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>https://plato.stanford.edu/entries/plato-ethics-politics/</t>
+          <t>https://www.gutenberg.org/ebooks/34901</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
+          <t>topic-freedom</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Wikipedia, "Negative liberty"</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Negative_liberty</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>topic-freedom</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Stanford Encyclopedia of Philosophy, 2014 version of the same entry (on the Stoics)</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/archives/sum2014/entries/liberty-positive-negative/</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>topic-freedom</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>The app's thoughts #15, #42, #168, #197, #198, and the others listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>topic-friendship-and-kindness</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Stanford Encyclopedia of Philosophy, "Friendship"</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/friendship/</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>topic-friendship-and-kindness</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Wikipedia, "Epicurus"</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Epicurus</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>topic-friendship-and-kindness</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Cambridge University Library, "Of friendship" (Montaigne exhibition)</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>https://wwwe.lib.cam.ac.uk/CUL/exhibitions/Montaigne/c3.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>topic-friendship-and-kindness</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Montaigne, "Of Friendship", Cotton translation (HyperEssays)</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>https://hyperessays.net/essays/on-friendship/</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>topic-friendship-and-kindness</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Wikipedia, "Michel de Montaigne"</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Michel_de_Montaigne</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>topic-friendship-and-kindness</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>The app's thoughts #58, #112, #115, #117, #211, #280, #502, #503, #511, and #512, with their sources</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>topic-habit-and-practice</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>The app's thoughts #22, #40, #109, #174, #311, #314, #338, #413, #432, #495, #514, and #527, with their sources</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>topic-happiness-and-the-good-life</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Stanford Encyclopedia of Philosophy, "Aristotle's Ethics"</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/aristotle-ethics/</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>topic-happiness-and-the-good-life</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>The app's thoughts #58, #64, #66, #67, #110, #116, #155, #158, #159, #331, and #479, with their sources</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
           <t>topic-justice</t>
         </is>
       </c>
-      <c r="B253" t="inlineStr">
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Wikipedia, "Justice"</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Justice</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>topic-justice</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Wikipedia, "Natural slavery"</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Natural_slavery</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>topic-justice</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Stanford Encyclopedia of Philosophy, "Justice"</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/justice/</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>topic-justice</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>"Epicurus"</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/epicurus/</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>topic-justice</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>"Plato's Ethics and Politics in The Republic"</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/plato-ethics-politics/</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>topic-justice</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
         <is>
           <t>The app's thoughts #71, #84, #85, #98, #127–129, #135, #491, #500, #504, and #617, with their sources</t>
         </is>
       </c>
-      <c r="C253" t="inlineStr"/>
+      <c r="C270" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>topic-law-and-rights</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Stanford Encyclopedia of Philosophy, "Locke's Political Philosophy"</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/locke-political/</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>topic-law-and-rights</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>"Aristotle's Political Theory"</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/aristotle-politics/</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>topic-law-and-rights</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>The app's thoughts listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>topic-learning-and-knowledge</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Stanford Encyclopedia of Philosophy, "Socrates"</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/socrates/</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>topic-learning-and-knowledge</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>"Laozi"</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/laozi/</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>topic-learning-and-knowledge</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>The app's thoughts #96, #97, #104, #162, #167, #175, #418, #420, #429, #470, #471, #480, and #482, with their sources</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>topic-love</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Stanford Encyclopedia of Philosophy, "Plato's Aesthetics"</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/plato-aesthetics/</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>topic-love</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>The app's thoughts #106, #219, #221, #280, #308, #378, #389, #559, #567, and #577, with their sources</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>topic-mind-and-emotions</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Stanford Encyclopedia of Philosophy, "Stoicism"</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/stoicism/</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>topic-mind-and-emotions</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>"Aristotle's Ethics"</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/aristotle-ethics/</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>topic-mind-and-emotions</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>"Hume's Moral Philosophy"</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/hume-moral/</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>topic-mind-and-emotions</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>The app's thoughts #7, #9, #111, #168, #169, #173, #228, #307, #308, and #315, with their sources</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>topic-nature-and-the-universe</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Stanford Encyclopedia of Philosophy, "Lucretius"</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/lucretius/</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>topic-nature-and-the-universe</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>"Stoicism"</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/stoicism/</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>topic-nature-and-the-universe</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>The app's thoughts #37, #44, #87, #89, #152, #226, #410, #422, #441, #543, and #553, with their sources</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>topic-purpose-and-meaning</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>The app's thoughts #116, #144, #163, #166, #214, #240, #243, #288, #296, #385, and #434, with their sources</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>topic-self-knowledge</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Stanford Encyclopedia of Philosophy, "Socrates"</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/socrates/</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>topic-self-knowledge</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>The app's thoughts #95, #214, #273, #283, #355, #364, #366, #493, and #513, with their sources</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>topic-solitude-and-stillness</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>The app's thoughts #3, #215, #225, #229, #230, #354, #417, #438, #522, and #541, with their sources</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>topic-suffering-and-resilience</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>The app's thoughts #6, #17, #28, #199, #213, #236, #248, #380, #555, #570, and #596, with their sources</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>topic-time-and-the-present</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>The app's thoughts #24, #26, #43, #63, #77, #79, #227, #278, #520, #579, and #583, with their sources</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr"/>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>topic-tolerance</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Stanford Encyclopedia of Philosophy, "Toleration"</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/toleration/</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>topic-tolerance</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Wikipedia, "A Letter Concerning Toleration"</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/A_Letter_Concerning_Toleration</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>topic-tolerance</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>"Treatise on Tolerance"</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Treatise_on_Tolerance</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>topic-tolerance</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>The app's thoughts listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>topic-war-and-peace</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Wikipedia, "Bhagavad Gita"</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Bhagavad_Gita</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>topic-war-and-peace</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>"The Kingdom of God Is Within You"</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/The_Kingdom_of_God_Is_Within_You</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>topic-war-and-peace</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Stanford Encyclopedia of Philosophy, "Hobbes's Moral and Political Philosophy"</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/hobbes-moral/</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>topic-war-and-peace</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>"Kant's Social and Political Philosophy"</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/kant-social-political/</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>topic-war-and-peace</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>The app's thoughts listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>topic-work-and-action</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>The app's thoughts #10, #12, #360, #368, #381, #432, #449, #472, and #611, with their sources</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>topic-work-and-wealth</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Wikipedia, "The Wealth of Nations"</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/The_Wealth_of_Nations</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>topic-work-and-wealth</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Stanford Encyclopedia of Philosophy, "Adam Smith's Moral and Political Philosophy"</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>https://plato.stanford.edu/entries/smith-moral-political/</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>topic-work-and-wealth</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>The app's thoughts listed above, with their sources</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>